<commit_message>
feat: add MProductionReport template for inventory reporting
</commit_message>
<xml_diff>
--- a/Eka_Report_back/MProductionReport.xlsx
+++ b/Eka_Report_back/MProductionReport.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Eka_Report_exe\Eka_Report_back\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\new\Eka_Report\Eka_Report_back\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F0233CF-82B3-45D6-B48C-128E241F37CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD46AC6D-2A7E-4DD3-9340-A7AB58817560}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5760" yWindow="3540" windowWidth="17280" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Manag Report" sheetId="12" r:id="rId1"/>
@@ -5458,7 +5458,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="151">
   <si>
     <t>MANAGEMENT PRODUCTION REPORT</t>
   </si>
@@ -5662,9 +5662,6 @@
   </si>
   <si>
     <t>CH-60</t>
-  </si>
-  <si>
-    <t xml:space="preserve">THE                                     </t>
   </si>
   <si>
     <t>Station Call</t>
@@ -6631,35 +6628,29 @@
     <xf numFmtId="1" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="27" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="28" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="26" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="18" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
@@ -6667,6 +6658,37 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="16" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -6685,57 +6707,32 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="27" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="28" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="18" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="26" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7067,52 +7064,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21">
-      <c r="A1" s="117" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="118"/>
-      <c r="C1" s="118"/>
-      <c r="D1" s="118"/>
-      <c r="E1" s="118"/>
-      <c r="F1" s="118"/>
-      <c r="G1" s="118"/>
-      <c r="H1" s="118"/>
-      <c r="I1" s="118"/>
-      <c r="J1" s="118"/>
-      <c r="K1" s="118"/>
-      <c r="L1" s="118"/>
-      <c r="M1" s="118"/>
-      <c r="N1" s="118"/>
-      <c r="O1" s="118"/>
-      <c r="P1" s="118"/>
-      <c r="Q1" s="118"/>
-      <c r="R1" s="118"/>
-      <c r="S1" s="118"/>
-      <c r="T1" s="118"/>
-      <c r="U1" s="119"/>
+      <c r="A1" s="76" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="77"/>
+      <c r="C1" s="77"/>
+      <c r="D1" s="77"/>
+      <c r="E1" s="77"/>
+      <c r="F1" s="77"/>
+      <c r="G1" s="77"/>
+      <c r="H1" s="77"/>
+      <c r="I1" s="77"/>
+      <c r="J1" s="77"/>
+      <c r="K1" s="77"/>
+      <c r="L1" s="77"/>
+      <c r="M1" s="77"/>
+      <c r="N1" s="77"/>
+      <c r="O1" s="77"/>
+      <c r="P1" s="77"/>
+      <c r="Q1" s="77"/>
+      <c r="R1" s="77"/>
+      <c r="S1" s="77"/>
+      <c r="T1" s="77"/>
+      <c r="U1" s="78"/>
     </row>
     <row r="2" spans="1:21" ht="15" customHeight="1" thickBot="1">
-      <c r="A2" s="120"/>
-      <c r="B2" s="121"/>
-      <c r="C2" s="121"/>
-      <c r="D2" s="121"/>
-      <c r="E2" s="121"/>
-      <c r="F2" s="121"/>
-      <c r="G2" s="121"/>
-      <c r="H2" s="121"/>
-      <c r="I2" s="121"/>
-      <c r="J2" s="121"/>
-      <c r="K2" s="121"/>
-      <c r="L2" s="121"/>
-      <c r="M2" s="121"/>
-      <c r="N2" s="121"/>
-      <c r="O2" s="121"/>
-      <c r="P2" s="121"/>
-      <c r="Q2" s="121"/>
-      <c r="R2" s="121"/>
-      <c r="S2" s="121"/>
-      <c r="T2" s="121"/>
-      <c r="U2" s="122"/>
+      <c r="A2" s="79"/>
+      <c r="B2" s="80"/>
+      <c r="C2" s="80"/>
+      <c r="D2" s="80"/>
+      <c r="E2" s="80"/>
+      <c r="F2" s="80"/>
+      <c r="G2" s="80"/>
+      <c r="H2" s="80"/>
+      <c r="I2" s="80"/>
+      <c r="J2" s="80"/>
+      <c r="K2" s="80"/>
+      <c r="L2" s="80"/>
+      <c r="M2" s="80"/>
+      <c r="N2" s="80"/>
+      <c r="O2" s="80"/>
+      <c r="P2" s="80"/>
+      <c r="Q2" s="80"/>
+      <c r="R2" s="80"/>
+      <c r="S2" s="80"/>
+      <c r="T2" s="80"/>
+      <c r="U2" s="81"/>
     </row>
     <row r="3" spans="1:21">
       <c r="A3" s="3"/>
@@ -7141,17 +7138,17 @@
       <c r="A4" s="67" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="124" t="s">
+      <c r="B4" s="83" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="82"/>
-      <c r="P4" s="105" t="s">
+      <c r="C4" s="74"/>
+      <c r="P4" s="82" t="s">
         <v>1</v>
       </c>
-      <c r="Q4" s="81"/>
-      <c r="R4" s="81"/>
-      <c r="S4" s="81"/>
-      <c r="T4" s="82"/>
+      <c r="Q4" s="73"/>
+      <c r="R4" s="73"/>
+      <c r="S4" s="73"/>
+      <c r="T4" s="74"/>
       <c r="U4" s="35" t="s">
         <v>2</v>
       </c>
@@ -7160,17 +7157,17 @@
       <c r="A5" s="67" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="116">
+      <c r="B5" s="75">
         <v>0.69398981410879634</v>
       </c>
-      <c r="C5" s="82"/>
-      <c r="P5" s="123" t="s">
+      <c r="C5" s="74"/>
+      <c r="P5" s="72" t="s">
         <v>3</v>
       </c>
-      <c r="Q5" s="81"/>
-      <c r="R5" s="81"/>
-      <c r="S5" s="81"/>
-      <c r="T5" s="82"/>
+      <c r="Q5" s="73"/>
+      <c r="R5" s="73"/>
+      <c r="S5" s="73"/>
+      <c r="T5" s="74"/>
       <c r="U5" s="6">
         <f>Daily!L3</f>
         <v>0</v>
@@ -7178,13 +7175,13 @@
     </row>
     <row r="6" spans="1:21">
       <c r="A6" s="5"/>
-      <c r="P6" s="123" t="s">
+      <c r="P6" s="72" t="s">
         <v>6</v>
       </c>
-      <c r="Q6" s="81"/>
-      <c r="R6" s="81"/>
-      <c r="S6" s="81"/>
-      <c r="T6" s="82"/>
+      <c r="Q6" s="73"/>
+      <c r="R6" s="73"/>
+      <c r="S6" s="73"/>
+      <c r="T6" s="74"/>
       <c r="U6" s="6">
         <f>Daily!M3</f>
         <v>0</v>
@@ -7197,33 +7194,33 @@
       <c r="U7" s="7"/>
     </row>
     <row r="8" spans="1:21">
-      <c r="A8" s="80"/>
-      <c r="B8" s="89"/>
-      <c r="C8" s="89"/>
-      <c r="D8" s="90"/>
-      <c r="E8" s="105" t="s">
+      <c r="A8" s="84"/>
+      <c r="B8" s="85"/>
+      <c r="C8" s="85"/>
+      <c r="D8" s="86"/>
+      <c r="E8" s="82" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="81"/>
-      <c r="G8" s="82"/>
+      <c r="F8" s="73"/>
+      <c r="G8" s="74"/>
       <c r="H8" s="59"/>
-      <c r="I8" s="105" t="s">
+      <c r="I8" s="82" t="s">
         <v>9</v>
       </c>
-      <c r="J8" s="81"/>
-      <c r="K8" s="81"/>
-      <c r="L8" s="81"/>
-      <c r="M8" s="82"/>
-      <c r="N8" s="105" t="s">
+      <c r="J8" s="73"/>
+      <c r="K8" s="73"/>
+      <c r="L8" s="73"/>
+      <c r="M8" s="74"/>
+      <c r="N8" s="82" t="s">
         <v>10</v>
       </c>
-      <c r="O8" s="81"/>
-      <c r="P8" s="82"/>
-      <c r="Q8" s="105" t="s">
+      <c r="O8" s="73"/>
+      <c r="P8" s="74"/>
+      <c r="Q8" s="82" t="s">
         <v>11</v>
       </c>
-      <c r="R8" s="81"/>
-      <c r="S8" s="82"/>
+      <c r="R8" s="73"/>
+      <c r="S8" s="74"/>
       <c r="T8" s="30" t="s">
         <v>12</v>
       </c>
@@ -7232,33 +7229,33 @@
       </c>
     </row>
     <row r="9" spans="1:21">
-      <c r="A9" s="91"/>
-      <c r="B9" s="92"/>
-      <c r="C9" s="92"/>
-      <c r="D9" s="93"/>
-      <c r="E9" s="111" t="s">
+      <c r="A9" s="87"/>
+      <c r="B9" s="88"/>
+      <c r="C9" s="88"/>
+      <c r="D9" s="89"/>
+      <c r="E9" s="90" t="s">
         <v>2</v>
       </c>
-      <c r="F9" s="81"/>
-      <c r="G9" s="82"/>
+      <c r="F9" s="73"/>
+      <c r="G9" s="74"/>
       <c r="H9" s="59"/>
-      <c r="I9" s="105" t="s">
+      <c r="I9" s="82" t="s">
         <v>14</v>
       </c>
-      <c r="J9" s="81"/>
-      <c r="K9" s="81"/>
-      <c r="L9" s="81"/>
-      <c r="M9" s="82"/>
-      <c r="N9" s="111" t="s">
+      <c r="J9" s="73"/>
+      <c r="K9" s="73"/>
+      <c r="L9" s="73"/>
+      <c r="M9" s="74"/>
+      <c r="N9" s="90" t="s">
         <v>15</v>
       </c>
-      <c r="O9" s="81"/>
-      <c r="P9" s="82"/>
-      <c r="Q9" s="111" t="s">
+      <c r="O9" s="73"/>
+      <c r="P9" s="74"/>
+      <c r="Q9" s="90" t="s">
         <v>16</v>
       </c>
-      <c r="R9" s="81"/>
-      <c r="S9" s="82"/>
+      <c r="R9" s="73"/>
+      <c r="S9" s="74"/>
       <c r="T9" s="30">
         <f>YTD!C12</f>
         <v>0</v>
@@ -7269,12 +7266,12 @@
       </c>
     </row>
     <row r="10" spans="1:21">
-      <c r="A10" s="88" t="s">
+      <c r="A10" s="91" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="81"/>
-      <c r="C10" s="81"/>
-      <c r="D10" s="82"/>
+      <c r="B10" s="73"/>
+      <c r="C10" s="73"/>
+      <c r="D10" s="74"/>
       <c r="E10" s="59" t="s">
         <v>18</v>
       </c>
@@ -7326,12 +7323,12 @@
       </c>
     </row>
     <row r="11" spans="1:21">
-      <c r="A11" s="114" t="s">
+      <c r="A11" s="92" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="81"/>
-      <c r="C11" s="81"/>
-      <c r="D11" s="82"/>
+      <c r="B11" s="73"/>
+      <c r="C11" s="73"/>
+      <c r="D11" s="74"/>
       <c r="E11" s="64">
         <v>70</v>
       </c>
@@ -7383,12 +7380,12 @@
       </c>
     </row>
     <row r="12" spans="1:21">
-      <c r="A12" s="115" t="s">
+      <c r="A12" s="93" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="81"/>
-      <c r="C12" s="81"/>
-      <c r="D12" s="82"/>
+      <c r="B12" s="73"/>
+      <c r="C12" s="73"/>
+      <c r="D12" s="74"/>
       <c r="E12" s="64">
         <v>80</v>
       </c>
@@ -7440,12 +7437,12 @@
       </c>
     </row>
     <row r="13" spans="1:21">
-      <c r="A13" s="115" t="s">
+      <c r="A13" s="93" t="s">
         <v>28</v>
       </c>
-      <c r="B13" s="81"/>
-      <c r="C13" s="81"/>
-      <c r="D13" s="82"/>
+      <c r="B13" s="73"/>
+      <c r="C13" s="73"/>
+      <c r="D13" s="74"/>
       <c r="E13" s="65">
         <f>Monthly!D4</f>
         <v>0</v>
@@ -7513,12 +7510,12 @@
       </c>
     </row>
     <row r="14" spans="1:21">
-      <c r="A14" s="115" t="s">
+      <c r="A14" s="93" t="s">
         <v>29</v>
       </c>
-      <c r="B14" s="81"/>
-      <c r="C14" s="81"/>
-      <c r="D14" s="82"/>
+      <c r="B14" s="73"/>
+      <c r="C14" s="73"/>
+      <c r="D14" s="74"/>
       <c r="E14" s="65">
         <f>Monthly!D5</f>
         <v>0</v>
@@ -7586,30 +7583,30 @@
       </c>
     </row>
     <row r="15" spans="1:21">
-      <c r="A15" s="80"/>
-      <c r="B15" s="82"/>
-      <c r="C15" s="111" t="s">
+      <c r="A15" s="84"/>
+      <c r="B15" s="74"/>
+      <c r="C15" s="90" t="s">
         <v>30</v>
       </c>
-      <c r="D15" s="82"/>
-      <c r="E15" s="111" t="s">
+      <c r="D15" s="74"/>
+      <c r="E15" s="90" t="s">
         <v>2</v>
       </c>
-      <c r="F15" s="81"/>
-      <c r="G15" s="81"/>
-      <c r="H15" s="82"/>
-      <c r="I15" s="105" t="s">
+      <c r="F15" s="73"/>
+      <c r="G15" s="73"/>
+      <c r="H15" s="74"/>
+      <c r="I15" s="82" t="s">
         <v>31</v>
       </c>
-      <c r="J15" s="81"/>
-      <c r="K15" s="81"/>
-      <c r="L15" s="81"/>
-      <c r="M15" s="82"/>
-      <c r="N15" s="111" t="s">
+      <c r="J15" s="73"/>
+      <c r="K15" s="73"/>
+      <c r="L15" s="73"/>
+      <c r="M15" s="74"/>
+      <c r="N15" s="90" t="s">
         <v>15</v>
       </c>
-      <c r="O15" s="81"/>
-      <c r="P15" s="82"/>
+      <c r="O15" s="73"/>
+      <c r="P15" s="74"/>
       <c r="Q15" s="11"/>
       <c r="R15" s="12"/>
       <c r="S15" s="12"/>
@@ -7617,8 +7614,8 @@
       <c r="U15" s="13"/>
     </row>
     <row r="16" spans="1:21">
-      <c r="A16" s="104"/>
-      <c r="B16" s="82"/>
+      <c r="A16" s="94"/>
+      <c r="B16" s="74"/>
       <c r="C16" s="33" t="s">
         <v>32</v>
       </c>
@@ -7763,7 +7760,7 @@
         <v>0</v>
       </c>
       <c r="J18" s="36" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K18" s="36">
         <v>0</v>
@@ -7775,10 +7772,10 @@
         <v>0</v>
       </c>
       <c r="N18" s="37" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="O18" s="37" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="P18" s="63">
         <f>SUM(N18:O18)</f>
@@ -7799,13 +7796,13 @@
       <c r="F19" s="8"/>
       <c r="G19" s="8"/>
       <c r="H19" s="8"/>
-      <c r="I19" s="105" t="s">
+      <c r="I19" s="82" t="s">
         <v>41</v>
       </c>
-      <c r="J19" s="81"/>
-      <c r="K19" s="81"/>
-      <c r="L19" s="81"/>
-      <c r="M19" s="82"/>
+      <c r="J19" s="73"/>
+      <c r="K19" s="73"/>
+      <c r="L19" s="73"/>
+      <c r="M19" s="74"/>
       <c r="N19" s="8"/>
       <c r="O19" s="8"/>
       <c r="P19" s="8"/>
@@ -7840,7 +7837,7 @@
         <v>0</v>
       </c>
       <c r="J21" s="36" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K21" s="36">
         <v>0</v>
@@ -7862,7 +7859,7 @@
         <v>0</v>
       </c>
       <c r="J22" s="36" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K22" s="36">
         <v>0</v>
@@ -7877,23 +7874,23 @@
     </row>
     <row r="23" spans="1:21">
       <c r="A23" s="5"/>
-      <c r="I23" s="105" t="s">
+      <c r="I23" s="82" t="s">
         <v>42</v>
       </c>
-      <c r="J23" s="81"/>
-      <c r="K23" s="81"/>
-      <c r="L23" s="81"/>
-      <c r="M23" s="82"/>
-      <c r="N23" s="112" t="s">
+      <c r="J23" s="73"/>
+      <c r="K23" s="73"/>
+      <c r="L23" s="73"/>
+      <c r="M23" s="74"/>
+      <c r="N23" s="100" t="s">
         <v>15</v>
       </c>
-      <c r="O23" s="81"/>
-      <c r="P23" s="82"/>
+      <c r="O23" s="73"/>
+      <c r="P23" s="74"/>
       <c r="U23" s="7"/>
     </row>
     <row r="24" spans="1:21">
-      <c r="A24" s="104"/>
-      <c r="B24" s="82"/>
+      <c r="A24" s="94"/>
+      <c r="B24" s="74"/>
       <c r="C24" s="59" t="s">
         <v>28</v>
       </c>
@@ -8089,13 +8086,13 @@
       <c r="F27" s="8"/>
       <c r="G27" s="8"/>
       <c r="H27" s="8"/>
-      <c r="I27" s="105" t="s">
+      <c r="I27" s="82" t="s">
         <v>45</v>
       </c>
-      <c r="J27" s="81"/>
-      <c r="K27" s="81"/>
-      <c r="L27" s="81"/>
-      <c r="M27" s="82"/>
+      <c r="J27" s="73"/>
+      <c r="K27" s="73"/>
+      <c r="L27" s="73"/>
+      <c r="M27" s="74"/>
       <c r="N27" s="8"/>
       <c r="O27" s="8"/>
       <c r="P27" s="8"/>
@@ -8184,15 +8181,15 @@
     </row>
     <row r="32" spans="1:21" ht="15.6">
       <c r="A32" s="5"/>
-      <c r="D32" s="113" t="s">
-        <v>150</v>
-      </c>
-      <c r="E32" s="113"/>
-      <c r="F32" s="113"/>
-      <c r="G32" s="113"/>
-      <c r="H32" s="113"/>
-      <c r="I32" s="113"/>
-      <c r="J32" s="113"/>
+      <c r="D32" s="101" t="s">
+        <v>149</v>
+      </c>
+      <c r="E32" s="101"/>
+      <c r="F32" s="101"/>
+      <c r="G32" s="101"/>
+      <c r="H32" s="101"/>
+      <c r="I32" s="101"/>
+      <c r="J32" s="101"/>
       <c r="K32" s="8"/>
       <c r="L32" s="8"/>
       <c r="M32" s="8"/>
@@ -8230,7 +8227,7 @@
     <row r="34" spans="1:25">
       <c r="A34" s="5"/>
       <c r="D34" s="27" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E34" s="25">
         <v>8.3000000000000007</v>
@@ -8258,36 +8255,36 @@
     <row r="35" spans="1:25">
       <c r="A35" s="5"/>
       <c r="H35" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="U35" s="7"/>
       <c r="V35" s="21"/>
       <c r="X35" s="8"/>
     </row>
     <row r="36" spans="1:25">
-      <c r="A36" s="106" t="s">
+      <c r="A36" s="95" t="s">
         <v>46</v>
       </c>
-      <c r="B36" s="81"/>
-      <c r="C36" s="81"/>
-      <c r="D36" s="81"/>
-      <c r="E36" s="81"/>
-      <c r="F36" s="81"/>
-      <c r="G36" s="81"/>
-      <c r="H36" s="81"/>
-      <c r="I36" s="81"/>
-      <c r="J36" s="81"/>
-      <c r="K36" s="81"/>
-      <c r="L36" s="81"/>
-      <c r="M36" s="81"/>
-      <c r="N36" s="81"/>
-      <c r="O36" s="81"/>
-      <c r="P36" s="81"/>
-      <c r="Q36" s="81"/>
-      <c r="R36" s="81"/>
-      <c r="S36" s="81"/>
-      <c r="T36" s="81"/>
-      <c r="U36" s="107"/>
+      <c r="B36" s="73"/>
+      <c r="C36" s="73"/>
+      <c r="D36" s="73"/>
+      <c r="E36" s="73"/>
+      <c r="F36" s="73"/>
+      <c r="G36" s="73"/>
+      <c r="H36" s="73"/>
+      <c r="I36" s="73"/>
+      <c r="J36" s="73"/>
+      <c r="K36" s="73"/>
+      <c r="L36" s="73"/>
+      <c r="M36" s="73"/>
+      <c r="N36" s="73"/>
+      <c r="O36" s="73"/>
+      <c r="P36" s="73"/>
+      <c r="Q36" s="73"/>
+      <c r="R36" s="73"/>
+      <c r="S36" s="73"/>
+      <c r="T36" s="73"/>
+      <c r="U36" s="96"/>
     </row>
     <row r="37" spans="1:25" s="1" customFormat="1" ht="43.2" customHeight="1">
       <c r="A37" s="60" t="s">
@@ -8311,11 +8308,11 @@
       <c r="G37" s="40" t="s">
         <v>59</v>
       </c>
-      <c r="H37" s="108" t="s">
+      <c r="H37" s="97" t="s">
         <v>60</v>
       </c>
-      <c r="I37" s="109"/>
-      <c r="J37" s="110"/>
+      <c r="I37" s="98"/>
+      <c r="J37" s="99"/>
       <c r="U37" s="7"/>
       <c r="V37" s="23"/>
       <c r="W37" s="24"/>
@@ -8344,9 +8341,9 @@
       <c r="G38" s="29">
         <v>0</v>
       </c>
-      <c r="H38" s="103"/>
-      <c r="I38" s="81"/>
-      <c r="J38" s="82"/>
+      <c r="H38" s="102"/>
+      <c r="I38" s="73"/>
+      <c r="J38" s="74"/>
       <c r="U38" s="7"/>
       <c r="V38" s="21"/>
       <c r="X38" s="8"/>
@@ -8373,9 +8370,9 @@
       <c r="G39" s="29">
         <v>0</v>
       </c>
-      <c r="H39" s="103"/>
-      <c r="I39" s="81"/>
-      <c r="J39" s="82"/>
+      <c r="H39" s="102"/>
+      <c r="I39" s="73"/>
+      <c r="J39" s="74"/>
       <c r="U39" s="7"/>
     </row>
     <row r="40" spans="1:25">
@@ -8400,9 +8397,9 @@
       <c r="G40" s="29">
         <v>0</v>
       </c>
-      <c r="H40" s="103"/>
-      <c r="I40" s="81"/>
-      <c r="J40" s="82"/>
+      <c r="H40" s="102"/>
+      <c r="I40" s="73"/>
+      <c r="J40" s="74"/>
       <c r="U40" s="7"/>
     </row>
     <row r="41" spans="1:25">
@@ -8427,9 +8424,9 @@
       <c r="G41" s="29">
         <v>0</v>
       </c>
-      <c r="H41" s="103"/>
-      <c r="I41" s="81"/>
-      <c r="J41" s="82"/>
+      <c r="H41" s="102"/>
+      <c r="I41" s="73"/>
+      <c r="J41" s="74"/>
       <c r="U41" s="7"/>
     </row>
     <row r="42" spans="1:25">
@@ -8454,9 +8451,9 @@
       <c r="G42" s="29">
         <v>0</v>
       </c>
-      <c r="H42" s="103"/>
-      <c r="I42" s="81"/>
-      <c r="J42" s="82"/>
+      <c r="H42" s="102"/>
+      <c r="I42" s="73"/>
+      <c r="J42" s="74"/>
       <c r="U42" s="7"/>
     </row>
     <row r="43" spans="1:25">
@@ -8481,11 +8478,9 @@
       <c r="G43" s="29">
         <v>0</v>
       </c>
-      <c r="H43" s="103" t="s">
-        <v>68</v>
-      </c>
-      <c r="I43" s="81"/>
-      <c r="J43" s="82"/>
+      <c r="H43" s="102"/>
+      <c r="I43" s="73"/>
+      <c r="J43" s="74"/>
       <c r="U43" s="7"/>
     </row>
     <row r="44" spans="1:25">
@@ -8493,109 +8488,109 @@
       <c r="U44" s="7"/>
     </row>
     <row r="45" spans="1:25">
-      <c r="A45" s="88" t="s">
+      <c r="A45" s="91" t="s">
+        <v>68</v>
+      </c>
+      <c r="B45" s="85"/>
+      <c r="C45" s="85"/>
+      <c r="D45" s="86"/>
+      <c r="E45" s="103">
+        <v>46182</v>
+      </c>
+      <c r="F45" s="73"/>
+      <c r="G45" s="73"/>
+      <c r="H45" s="73"/>
+      <c r="I45" s="73"/>
+      <c r="J45" s="73"/>
+      <c r="K45" s="73"/>
+      <c r="L45" s="73"/>
+      <c r="M45" s="73"/>
+      <c r="N45" s="74"/>
+      <c r="O45" s="104"/>
+      <c r="P45" s="85"/>
+      <c r="Q45" s="85"/>
+      <c r="R45" s="85"/>
+      <c r="S45" s="85"/>
+      <c r="T45" s="85"/>
+      <c r="U45" s="105"/>
+    </row>
+    <row r="46" spans="1:25">
+      <c r="A46" s="87"/>
+      <c r="B46" s="88"/>
+      <c r="C46" s="88"/>
+      <c r="D46" s="89"/>
+      <c r="E46" s="108" t="s">
         <v>69</v>
       </c>
-      <c r="B45" s="89"/>
-      <c r="C45" s="89"/>
-      <c r="D45" s="90"/>
-      <c r="E45" s="94">
-        <v>46182</v>
-      </c>
-      <c r="F45" s="81"/>
-      <c r="G45" s="81"/>
-      <c r="H45" s="81"/>
-      <c r="I45" s="81"/>
-      <c r="J45" s="81"/>
-      <c r="K45" s="81"/>
-      <c r="L45" s="81"/>
-      <c r="M45" s="81"/>
-      <c r="N45" s="82"/>
-      <c r="O45" s="95"/>
-      <c r="P45" s="89"/>
-      <c r="Q45" s="89"/>
-      <c r="R45" s="89"/>
-      <c r="S45" s="89"/>
-      <c r="T45" s="89"/>
-      <c r="U45" s="96"/>
-    </row>
-    <row r="46" spans="1:25">
-      <c r="A46" s="91"/>
-      <c r="B46" s="92"/>
-      <c r="C46" s="92"/>
-      <c r="D46" s="93"/>
-      <c r="E46" s="99" t="s">
+      <c r="F46" s="73"/>
+      <c r="G46" s="73"/>
+      <c r="H46" s="73"/>
+      <c r="I46" s="73"/>
+      <c r="J46" s="73"/>
+      <c r="K46" s="73"/>
+      <c r="L46" s="73"/>
+      <c r="M46" s="73"/>
+      <c r="N46" s="74"/>
+      <c r="O46" s="106"/>
+      <c r="P46" s="88"/>
+      <c r="Q46" s="88"/>
+      <c r="R46" s="88"/>
+      <c r="S46" s="88"/>
+      <c r="T46" s="88"/>
+      <c r="U46" s="107"/>
+    </row>
+    <row r="47" spans="1:25" s="2" customFormat="1">
+      <c r="A47" s="109" t="s">
         <v>70</v>
       </c>
-      <c r="F46" s="81"/>
-      <c r="G46" s="81"/>
-      <c r="H46" s="81"/>
-      <c r="I46" s="81"/>
-      <c r="J46" s="81"/>
-      <c r="K46" s="81"/>
-      <c r="L46" s="81"/>
-      <c r="M46" s="81"/>
-      <c r="N46" s="82"/>
-      <c r="O46" s="97"/>
-      <c r="P46" s="92"/>
-      <c r="Q46" s="92"/>
-      <c r="R46" s="92"/>
-      <c r="S46" s="92"/>
-      <c r="T46" s="92"/>
-      <c r="U46" s="98"/>
-    </row>
-    <row r="47" spans="1:25" s="2" customFormat="1">
-      <c r="A47" s="100" t="s">
-        <v>71</v>
-      </c>
-      <c r="B47" s="81"/>
-      <c r="C47" s="81"/>
-      <c r="D47" s="82"/>
+      <c r="B47" s="73"/>
+      <c r="C47" s="73"/>
+      <c r="D47" s="74"/>
       <c r="E47" s="62" t="s">
         <v>38</v>
       </c>
       <c r="F47" s="62" t="s">
+        <v>71</v>
+      </c>
+      <c r="G47" s="61" t="s">
         <v>72</v>
       </c>
-      <c r="G47" s="61" t="s">
+      <c r="H47" s="61" t="s">
         <v>73</v>
       </c>
-      <c r="H47" s="61" t="s">
+      <c r="I47" s="61" t="s">
         <v>74</v>
       </c>
-      <c r="I47" s="61" t="s">
+      <c r="J47" s="61" t="s">
         <v>75</v>
       </c>
-      <c r="J47" s="61" t="s">
+      <c r="K47" s="110" t="s">
         <v>76</v>
       </c>
-      <c r="K47" s="101" t="s">
+      <c r="L47" s="111"/>
+      <c r="M47" s="110" t="s">
         <v>77</v>
       </c>
-      <c r="L47" s="85"/>
-      <c r="M47" s="101" t="s">
+      <c r="N47" s="111"/>
+      <c r="O47" s="112" t="s">
         <v>78</v>
       </c>
-      <c r="N47" s="85"/>
-      <c r="O47" s="102" t="s">
+      <c r="P47" s="113"/>
+      <c r="Q47" s="113"/>
+      <c r="R47" s="111"/>
+      <c r="S47" s="110" t="s">
         <v>79</v>
       </c>
-      <c r="P47" s="84"/>
-      <c r="Q47" s="84"/>
-      <c r="R47" s="85"/>
-      <c r="S47" s="101" t="s">
+      <c r="T47" s="113"/>
+      <c r="U47" s="114"/>
+    </row>
+    <row r="48" spans="1:25">
+      <c r="A48" s="84" t="s">
         <v>80</v>
       </c>
-      <c r="T47" s="84"/>
-      <c r="U47" s="87"/>
-    </row>
-    <row r="48" spans="1:25">
-      <c r="A48" s="80" t="s">
-        <v>81</v>
-      </c>
-      <c r="B48" s="81"/>
-      <c r="C48" s="81"/>
-      <c r="D48" s="82"/>
+      <c r="B48" s="73"/>
+      <c r="C48" s="73"/>
+      <c r="D48" s="74"/>
       <c r="E48" s="65">
         <f>'Line Stop_Prod Loss'!G5</f>
         <v>0.5</v>
@@ -8632,23 +8627,21 @@
       <c r="N48" s="65">
         <v>0</v>
       </c>
-      <c r="O48" s="83" t="s">
+      <c r="O48" s="115"/>
+      <c r="P48" s="113"/>
+      <c r="Q48" s="113"/>
+      <c r="R48" s="111"/>
+      <c r="S48" s="116"/>
+      <c r="T48" s="113"/>
+      <c r="U48" s="114"/>
+    </row>
+    <row r="49" spans="1:21">
+      <c r="A49" s="84" t="s">
         <v>82</v>
       </c>
-      <c r="P48" s="84"/>
-      <c r="Q48" s="84"/>
-      <c r="R48" s="85"/>
-      <c r="S48" s="86"/>
-      <c r="T48" s="84"/>
-      <c r="U48" s="87"/>
-    </row>
-    <row r="49" spans="1:21">
-      <c r="A49" s="80" t="s">
-        <v>83</v>
-      </c>
-      <c r="B49" s="81"/>
-      <c r="C49" s="81"/>
-      <c r="D49" s="82"/>
+      <c r="B49" s="73"/>
+      <c r="C49" s="73"/>
+      <c r="D49" s="74"/>
       <c r="E49" s="28">
         <f>'Line Stop_Prod Loss'!G6</f>
         <v>156.30000000000001</v>
@@ -8685,23 +8678,21 @@
       <c r="N49" s="28">
         <v>0</v>
       </c>
-      <c r="O49" s="83" t="s">
+      <c r="O49" s="115"/>
+      <c r="P49" s="113"/>
+      <c r="Q49" s="113"/>
+      <c r="R49" s="111"/>
+      <c r="S49" s="116"/>
+      <c r="T49" s="113"/>
+      <c r="U49" s="114"/>
+    </row>
+    <row r="50" spans="1:21">
+      <c r="A50" s="84" t="s">
         <v>84</v>
       </c>
-      <c r="P49" s="84"/>
-      <c r="Q49" s="84"/>
-      <c r="R49" s="85"/>
-      <c r="S49" s="86"/>
-      <c r="T49" s="84"/>
-      <c r="U49" s="87"/>
-    </row>
-    <row r="50" spans="1:21">
-      <c r="A50" s="80" t="s">
-        <v>85</v>
-      </c>
-      <c r="B50" s="81"/>
-      <c r="C50" s="81"/>
-      <c r="D50" s="82"/>
+      <c r="B50" s="73"/>
+      <c r="C50" s="73"/>
+      <c r="D50" s="74"/>
       <c r="E50" s="28">
         <f>'Line Stop_Prod Loss'!G7</f>
         <v>0</v>
@@ -8738,21 +8729,21 @@
       <c r="N50" s="28">
         <v>0</v>
       </c>
-      <c r="O50" s="83"/>
-      <c r="P50" s="84"/>
-      <c r="Q50" s="84"/>
-      <c r="R50" s="85"/>
-      <c r="S50" s="86"/>
-      <c r="T50" s="84"/>
-      <c r="U50" s="87"/>
+      <c r="O50" s="115"/>
+      <c r="P50" s="113"/>
+      <c r="Q50" s="113"/>
+      <c r="R50" s="111"/>
+      <c r="S50" s="116"/>
+      <c r="T50" s="113"/>
+      <c r="U50" s="114"/>
     </row>
     <row r="51" spans="1:21">
-      <c r="A51" s="80" t="s">
-        <v>86</v>
-      </c>
-      <c r="B51" s="81"/>
-      <c r="C51" s="81"/>
-      <c r="D51" s="82"/>
+      <c r="A51" s="84" t="s">
+        <v>85</v>
+      </c>
+      <c r="B51" s="73"/>
+      <c r="C51" s="73"/>
+      <c r="D51" s="74"/>
       <c r="E51" s="28">
         <f>'Line Stop_Prod Loss'!G8</f>
         <v>0.1</v>
@@ -8789,23 +8780,21 @@
       <c r="N51" s="28">
         <v>0</v>
       </c>
-      <c r="O51" s="83" t="s">
+      <c r="O51" s="115"/>
+      <c r="P51" s="113"/>
+      <c r="Q51" s="113"/>
+      <c r="R51" s="111"/>
+      <c r="S51" s="116"/>
+      <c r="T51" s="113"/>
+      <c r="U51" s="114"/>
+    </row>
+    <row r="52" spans="1:21" ht="15" customHeight="1" thickBot="1">
+      <c r="A52" s="117" t="s">
         <v>87</v>
       </c>
-      <c r="P51" s="84"/>
-      <c r="Q51" s="84"/>
-      <c r="R51" s="85"/>
-      <c r="S51" s="86"/>
-      <c r="T51" s="84"/>
-      <c r="U51" s="87"/>
-    </row>
-    <row r="52" spans="1:21" ht="15" customHeight="1" thickBot="1">
-      <c r="A52" s="72" t="s">
-        <v>88</v>
-      </c>
-      <c r="B52" s="73"/>
-      <c r="C52" s="73"/>
-      <c r="D52" s="74"/>
+      <c r="B52" s="118"/>
+      <c r="C52" s="118"/>
+      <c r="D52" s="119"/>
       <c r="E52" s="68">
         <f>'Line Stop_Prod Loss'!G9</f>
         <v>0</v>
@@ -8842,39 +8831,49 @@
       <c r="N52" s="68">
         <v>0</v>
       </c>
-      <c r="O52" s="75"/>
-      <c r="P52" s="76"/>
-      <c r="Q52" s="76"/>
-      <c r="R52" s="77"/>
-      <c r="S52" s="78"/>
-      <c r="T52" s="76"/>
-      <c r="U52" s="79"/>
+      <c r="O52" s="120"/>
+      <c r="P52" s="121"/>
+      <c r="Q52" s="121"/>
+      <c r="R52" s="122"/>
+      <c r="S52" s="123"/>
+      <c r="T52" s="121"/>
+      <c r="U52" s="124"/>
     </row>
     <row r="53" spans="1:21">
       <c r="L53" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="64">
-    <mergeCell ref="P6:T6"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="A1:U2"/>
-    <mergeCell ref="P4:T4"/>
-    <mergeCell ref="P5:T5"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="A8:D9"/>
-    <mergeCell ref="E8:G8"/>
-    <mergeCell ref="I8:M8"/>
-    <mergeCell ref="N8:P8"/>
-    <mergeCell ref="Q8:S8"/>
-    <mergeCell ref="E9:G9"/>
-    <mergeCell ref="I9:M9"/>
-    <mergeCell ref="N9:P9"/>
-    <mergeCell ref="Q9:S9"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="A13:D13"/>
-    <mergeCell ref="A14:D14"/>
+    <mergeCell ref="A52:D52"/>
+    <mergeCell ref="O52:R52"/>
+    <mergeCell ref="S52:U52"/>
+    <mergeCell ref="A50:D50"/>
+    <mergeCell ref="O50:R50"/>
+    <mergeCell ref="S50:U50"/>
+    <mergeCell ref="A51:D51"/>
+    <mergeCell ref="O51:R51"/>
+    <mergeCell ref="S51:U51"/>
+    <mergeCell ref="A48:D48"/>
+    <mergeCell ref="O48:R48"/>
+    <mergeCell ref="S48:U48"/>
+    <mergeCell ref="A49:D49"/>
+    <mergeCell ref="O49:R49"/>
+    <mergeCell ref="S49:U49"/>
+    <mergeCell ref="A45:D46"/>
+    <mergeCell ref="E45:N45"/>
+    <mergeCell ref="O45:U46"/>
+    <mergeCell ref="E46:N46"/>
+    <mergeCell ref="A47:D47"/>
+    <mergeCell ref="K47:L47"/>
+    <mergeCell ref="M47:N47"/>
+    <mergeCell ref="O47:R47"/>
+    <mergeCell ref="S47:U47"/>
+    <mergeCell ref="H42:J42"/>
+    <mergeCell ref="H43:J43"/>
+    <mergeCell ref="H40:J40"/>
+    <mergeCell ref="H41:J41"/>
+    <mergeCell ref="H38:J38"/>
+    <mergeCell ref="H39:J39"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="I27:M27"/>
     <mergeCell ref="A36:U36"/>
@@ -8889,36 +8888,26 @@
     <mergeCell ref="A15:B15"/>
     <mergeCell ref="C15:D15"/>
     <mergeCell ref="D32:J32"/>
-    <mergeCell ref="H42:J42"/>
-    <mergeCell ref="H43:J43"/>
-    <mergeCell ref="H40:J40"/>
-    <mergeCell ref="H41:J41"/>
-    <mergeCell ref="H38:J38"/>
-    <mergeCell ref="H39:J39"/>
-    <mergeCell ref="A45:D46"/>
-    <mergeCell ref="E45:N45"/>
-    <mergeCell ref="O45:U46"/>
-    <mergeCell ref="E46:N46"/>
-    <mergeCell ref="A47:D47"/>
-    <mergeCell ref="K47:L47"/>
-    <mergeCell ref="M47:N47"/>
-    <mergeCell ref="O47:R47"/>
-    <mergeCell ref="S47:U47"/>
-    <mergeCell ref="A48:D48"/>
-    <mergeCell ref="O48:R48"/>
-    <mergeCell ref="S48:U48"/>
-    <mergeCell ref="A49:D49"/>
-    <mergeCell ref="O49:R49"/>
-    <mergeCell ref="S49:U49"/>
-    <mergeCell ref="A52:D52"/>
-    <mergeCell ref="O52:R52"/>
-    <mergeCell ref="S52:U52"/>
-    <mergeCell ref="A50:D50"/>
-    <mergeCell ref="O50:R50"/>
-    <mergeCell ref="S50:U50"/>
-    <mergeCell ref="A51:D51"/>
-    <mergeCell ref="O51:R51"/>
-    <mergeCell ref="S51:U51"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="A14:D14"/>
+    <mergeCell ref="A8:D9"/>
+    <mergeCell ref="E8:G8"/>
+    <mergeCell ref="I8:M8"/>
+    <mergeCell ref="N8:P8"/>
+    <mergeCell ref="Q8:S8"/>
+    <mergeCell ref="E9:G9"/>
+    <mergeCell ref="I9:M9"/>
+    <mergeCell ref="N9:P9"/>
+    <mergeCell ref="Q9:S9"/>
+    <mergeCell ref="P6:T6"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="A1:U2"/>
+    <mergeCell ref="P4:T4"/>
+    <mergeCell ref="P5:T5"/>
+    <mergeCell ref="B4:C4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="49" orientation="landscape" r:id="rId1"/>
@@ -8940,87 +8929,87 @@
   <sheetData>
     <row r="1" spans="2:13">
       <c r="B1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2" spans="2:13">
       <c r="C2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D2" t="s">
         <v>90</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>91</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>92</v>
       </c>
-      <c r="F2" t="s">
+      <c r="L2" t="s">
         <v>93</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>94</v>
-      </c>
-      <c r="M2" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="3" spans="2:13"/>
     <row r="11" spans="2:13">
       <c r="B11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="12" spans="2:13">
       <c r="C12" t="s">
+        <v>89</v>
+      </c>
+      <c r="D12" t="s">
         <v>90</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>91</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
         <v>92</v>
-      </c>
-      <c r="F12" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="13" spans="2:13"/>
     <row r="20" spans="2:6">
       <c r="B20" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="21" spans="2:6">
       <c r="C21" t="s">
+        <v>89</v>
+      </c>
+      <c r="D21" t="s">
         <v>90</v>
       </c>
-      <c r="D21" t="s">
+      <c r="E21" t="s">
         <v>91</v>
       </c>
-      <c r="E21" t="s">
+      <c r="F21" t="s">
         <v>92</v>
-      </c>
-      <c r="F21" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="22" spans="2:6"/>
     <row r="30" spans="2:6">
       <c r="B30" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="31" spans="2:6">
       <c r="C31" t="s">
+        <v>89</v>
+      </c>
+      <c r="D31" t="s">
         <v>90</v>
       </c>
-      <c r="D31" t="s">
+      <c r="E31" t="s">
         <v>91</v>
       </c>
-      <c r="E31" t="s">
+      <c r="F31" t="s">
         <v>92</v>
-      </c>
-      <c r="F31" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="32" spans="2:6"/>
@@ -9044,7 +9033,7 @@
   <sheetData>
     <row r="2" spans="1:15">
       <c r="B2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -9052,51 +9041,51 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
+        <v>99</v>
+      </c>
+      <c r="C4" t="s">
         <v>100</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>101</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>102</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>103</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>104</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>105</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>106</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>107</v>
       </c>
-      <c r="J4" t="s">
+      <c r="K4" t="s">
         <v>108</v>
       </c>
-      <c r="K4" t="s">
+      <c r="L4" t="s">
         <v>109</v>
       </c>
-      <c r="L4" t="s">
+      <c r="M4" t="s">
         <v>110</v>
       </c>
-      <c r="M4" t="s">
+      <c r="N4" t="s">
         <v>111</v>
       </c>
-      <c r="N4" t="s">
+      <c r="O4" t="s">
         <v>112</v>
-      </c>
-      <c r="O4" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="5" spans="1:15">
       <c r="B5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -9120,12 +9109,12 @@
         <v>74.099999999999994</v>
       </c>
       <c r="N5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="6" spans="1:15">
       <c r="B6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -9149,12 +9138,12 @@
         <v>156.30000000000001</v>
       </c>
       <c r="N6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="7" spans="1:15">
       <c r="B7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -9180,7 +9169,7 @@
     </row>
     <row r="8" spans="1:15">
       <c r="B8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -9204,12 +9193,12 @@
         <v>0.2</v>
       </c>
       <c r="N8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="9" spans="1:15">
       <c r="B9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C9">
         <v>0</v>
@@ -9235,7 +9224,7 @@
     </row>
     <row r="21" spans="1:15">
       <c r="B21" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="23" spans="1:15">
@@ -9243,51 +9232,51 @@
         <v>2</v>
       </c>
       <c r="B23" t="s">
+        <v>99</v>
+      </c>
+      <c r="C23" t="s">
         <v>100</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
         <v>101</v>
       </c>
-      <c r="D23" t="s">
+      <c r="E23" t="s">
         <v>102</v>
       </c>
-      <c r="E23" t="s">
+      <c r="F23" t="s">
         <v>103</v>
       </c>
-      <c r="F23" t="s">
+      <c r="G23" t="s">
         <v>104</v>
       </c>
-      <c r="G23" t="s">
+      <c r="H23" t="s">
         <v>105</v>
       </c>
-      <c r="H23" t="s">
+      <c r="I23" t="s">
         <v>106</v>
       </c>
-      <c r="I23" t="s">
+      <c r="J23" t="s">
         <v>107</v>
       </c>
-      <c r="J23" t="s">
+      <c r="K23" t="s">
         <v>108</v>
       </c>
-      <c r="K23" t="s">
+      <c r="L23" t="s">
         <v>109</v>
       </c>
-      <c r="L23" t="s">
+      <c r="M23" t="s">
         <v>110</v>
       </c>
-      <c r="M23" t="s">
+      <c r="N23" t="s">
         <v>111</v>
       </c>
-      <c r="N23" t="s">
+      <c r="O23" t="s">
         <v>112</v>
-      </c>
-      <c r="O23" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="24" spans="1:15">
       <c r="B24" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C24">
         <v>0</v>
@@ -9311,15 +9300,15 @@
         <v>994.4</v>
       </c>
       <c r="N24" t="s">
+        <v>114</v>
+      </c>
+      <c r="O24" t="s">
         <v>115</v>
-      </c>
-      <c r="O24" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="25" spans="1:15">
       <c r="B25" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C25">
         <v>0</v>
@@ -9343,15 +9332,15 @@
         <v>1308.9000000000001</v>
       </c>
       <c r="N25" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O25" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="26" spans="1:15">
       <c r="B26" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C26">
         <v>0</v>
@@ -9375,15 +9364,15 @@
         <v>111.8</v>
       </c>
       <c r="N26" t="s">
+        <v>116</v>
+      </c>
+      <c r="O26" t="s">
         <v>117</v>
-      </c>
-      <c r="O26" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="27" spans="1:15">
       <c r="B27" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C27">
         <v>0</v>
@@ -9407,15 +9396,15 @@
         <v>13</v>
       </c>
       <c r="N27" t="s">
+        <v>118</v>
+      </c>
+      <c r="O27" t="s">
         <v>119</v>
-      </c>
-      <c r="O27" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="28" spans="1:15">
       <c r="B28" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C28">
         <v>0</v>
@@ -9441,7 +9430,7 @@
     </row>
     <row r="41" spans="1:13">
       <c r="B41" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="43" spans="1:13">
@@ -9464,165 +9453,165 @@
   <sheetData>
     <row r="1" spans="2:13">
       <c r="B1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2" spans="2:13">
       <c r="C2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D2" t="s">
         <v>122</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>123</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>124</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>125</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>126</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>127</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>128</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>129</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>130</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>131</v>
-      </c>
-      <c r="M2" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="3" spans="2:13"/>
     <row r="10" spans="2:13">
       <c r="B10" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="11" spans="2:13">
       <c r="C11" t="s">
+        <v>121</v>
+      </c>
+      <c r="D11" t="s">
         <v>122</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>123</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
         <v>124</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>125</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>126</v>
       </c>
-      <c r="H11" t="s">
+      <c r="I11" t="s">
         <v>127</v>
       </c>
-      <c r="I11" t="s">
+      <c r="J11" t="s">
         <v>128</v>
       </c>
-      <c r="J11" t="s">
+      <c r="K11" t="s">
         <v>129</v>
       </c>
-      <c r="K11" t="s">
+      <c r="L11" t="s">
         <v>130</v>
       </c>
-      <c r="L11" t="s">
+      <c r="M11" t="s">
         <v>131</v>
-      </c>
-      <c r="M11" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="12" spans="2:13"/>
     <row r="20" spans="2:13">
       <c r="B20" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="21" spans="2:13">
       <c r="C21" t="s">
+        <v>121</v>
+      </c>
+      <c r="D21" t="s">
         <v>122</v>
       </c>
-      <c r="D21" t="s">
+      <c r="E21" t="s">
         <v>123</v>
       </c>
-      <c r="E21" t="s">
+      <c r="F21" t="s">
         <v>124</v>
       </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
         <v>125</v>
       </c>
-      <c r="G21" t="s">
+      <c r="H21" t="s">
         <v>126</v>
       </c>
-      <c r="H21" t="s">
+      <c r="I21" t="s">
         <v>127</v>
       </c>
-      <c r="I21" t="s">
+      <c r="J21" t="s">
         <v>128</v>
       </c>
-      <c r="J21" t="s">
+      <c r="K21" t="s">
         <v>129</v>
       </c>
-      <c r="K21" t="s">
+      <c r="L21" t="s">
         <v>130</v>
       </c>
-      <c r="L21" t="s">
+      <c r="M21" t="s">
         <v>131</v>
-      </c>
-      <c r="M21" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="22" spans="2:13"/>
     <row r="30" spans="2:13">
       <c r="B30" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="31" spans="2:13">
       <c r="C31" t="s">
+        <v>121</v>
+      </c>
+      <c r="D31" t="s">
         <v>122</v>
       </c>
-      <c r="D31" t="s">
+      <c r="E31" t="s">
         <v>123</v>
       </c>
-      <c r="E31" t="s">
+      <c r="F31" t="s">
         <v>124</v>
       </c>
-      <c r="F31" t="s">
+      <c r="G31" t="s">
         <v>125</v>
       </c>
-      <c r="G31" t="s">
+      <c r="H31" t="s">
         <v>126</v>
       </c>
-      <c r="H31" t="s">
+      <c r="I31" t="s">
         <v>127</v>
       </c>
-      <c r="I31" t="s">
+      <c r="J31" t="s">
         <v>128</v>
       </c>
-      <c r="J31" t="s">
+      <c r="K31" t="s">
         <v>129</v>
       </c>
-      <c r="K31" t="s">
+      <c r="L31" t="s">
         <v>130</v>
       </c>
-      <c r="L31" t="s">
+      <c r="M31" t="s">
         <v>131</v>
-      </c>
-      <c r="M31" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="32" spans="2:13"/>
@@ -9640,81 +9629,81 @@
   <sheetData>
     <row r="1" spans="2:6">
       <c r="B1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2" spans="2:6">
       <c r="C2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D2" t="s">
         <v>133</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>134</v>
       </c>
-      <c r="E2" t="s">
-        <v>135</v>
-      </c>
       <c r="F2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3" spans="2:6"/>
     <row r="10" spans="2:6">
       <c r="B10" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="11" spans="2:6">
       <c r="C11" t="s">
+        <v>132</v>
+      </c>
+      <c r="D11" t="s">
         <v>133</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>134</v>
       </c>
-      <c r="E11" t="s">
-        <v>135</v>
-      </c>
       <c r="F11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="12" spans="2:6"/>
     <row r="20" spans="2:6">
       <c r="B20" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="21" spans="2:6">
       <c r="C21" t="s">
+        <v>132</v>
+      </c>
+      <c r="D21" t="s">
         <v>133</v>
       </c>
-      <c r="D21" t="s">
+      <c r="E21" t="s">
         <v>134</v>
       </c>
-      <c r="E21" t="s">
-        <v>135</v>
-      </c>
       <c r="F21" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="22" spans="2:6"/>
     <row r="30" spans="2:6">
       <c r="B30" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="31" spans="2:6">
       <c r="C31" t="s">
+        <v>132</v>
+      </c>
+      <c r="D31" t="s">
         <v>133</v>
       </c>
-      <c r="D31" t="s">
+      <c r="E31" t="s">
         <v>134</v>
       </c>
-      <c r="E31" t="s">
-        <v>135</v>
-      </c>
       <c r="F31" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="32" spans="2:6"/>
@@ -9732,41 +9721,41 @@
   <sheetData>
     <row r="1" spans="2:6">
       <c r="B1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2" spans="2:6">
       <c r="C2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D2" t="s">
         <v>136</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>137</v>
       </c>
-      <c r="E2" t="s">
-        <v>138</v>
-      </c>
       <c r="F2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3" spans="2:6"/>
     <row r="10" spans="2:6">
       <c r="B10" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="11" spans="2:6">
       <c r="C11" t="s">
+        <v>135</v>
+      </c>
+      <c r="D11" t="s">
         <v>136</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>137</v>
       </c>
-      <c r="E11" t="s">
-        <v>138</v>
-      </c>
       <c r="F11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="12" spans="2:6"/>
@@ -9784,26 +9773,26 @@
   <sheetData>
     <row r="1" spans="2:8">
       <c r="B1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2" spans="2:8">
       <c r="C2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D2" t="s">
         <v>139</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>140</v>
       </c>
-      <c r="E2" t="s">
-        <v>141</v>
-      </c>
       <c r="F2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3" spans="2:8">
       <c r="B3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H3" t="str">
         <f>_xlfn.CONCAT(B3,C3)</f>
@@ -9812,26 +9801,26 @@
     </row>
     <row r="10" spans="2:8">
       <c r="B10" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="11" spans="2:8">
       <c r="C11" t="s">
+        <v>138</v>
+      </c>
+      <c r="D11" t="s">
         <v>139</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>140</v>
       </c>
-      <c r="E11" t="s">
-        <v>141</v>
-      </c>
       <c r="F11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="12" spans="2:8">
       <c r="B12" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="H12" t="str">
         <f>_xlfn.CONCAT(B12,C12)</f>
@@ -9840,41 +9829,41 @@
     </row>
     <row r="20" spans="2:6">
       <c r="B20" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="21" spans="2:6">
       <c r="C21" t="s">
+        <v>138</v>
+      </c>
+      <c r="D21" t="s">
         <v>139</v>
       </c>
-      <c r="D21" t="s">
+      <c r="E21" t="s">
         <v>140</v>
       </c>
-      <c r="E21" t="s">
-        <v>141</v>
-      </c>
       <c r="F21" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="22" spans="2:6"/>
     <row r="30" spans="2:6">
       <c r="B30" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="31" spans="2:6">
       <c r="C31" t="s">
+        <v>138</v>
+      </c>
+      <c r="D31" t="s">
         <v>139</v>
       </c>
-      <c r="D31" t="s">
+      <c r="E31" t="s">
         <v>140</v>
       </c>
-      <c r="E31" t="s">
-        <v>141</v>
-      </c>
       <c r="F31" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="32" spans="2:6"/>
@@ -9892,29 +9881,29 @@
   <sheetData>
     <row r="1" spans="2:8">
       <c r="B1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2" spans="2:8">
       <c r="C2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D2" t="s">
         <v>144</v>
       </c>
-      <c r="D2" t="s">
-        <v>145</v>
-      </c>
       <c r="E2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3" spans="2:8">
       <c r="B3" t="s">
+        <v>145</v>
+      </c>
+      <c r="C3" t="s">
         <v>146</v>
-      </c>
-      <c r="C3" t="s">
-        <v>147</v>
       </c>
       <c r="D3">
         <v>88</v>
@@ -9933,29 +9922,29 @@
     </row>
     <row r="10" spans="2:8">
       <c r="B10" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="11" spans="2:8">
       <c r="C11" t="s">
+        <v>143</v>
+      </c>
+      <c r="D11" t="s">
         <v>144</v>
       </c>
-      <c r="D11" t="s">
-        <v>145</v>
-      </c>
       <c r="E11" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="12" spans="2:8">
       <c r="B12" t="s">
+        <v>145</v>
+      </c>
+      <c r="C12" t="s">
         <v>146</v>
-      </c>
-      <c r="C12" t="s">
-        <v>147</v>
       </c>
       <c r="D12">
         <v>88</v>
@@ -9970,29 +9959,29 @@
     </row>
     <row r="20" spans="2:6">
       <c r="B20" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="21" spans="2:6">
       <c r="C21" t="s">
+        <v>143</v>
+      </c>
+      <c r="D21" t="s">
         <v>144</v>
       </c>
-      <c r="D21" t="s">
-        <v>145</v>
-      </c>
       <c r="E21" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F21" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="22" spans="2:6">
       <c r="B22" t="s">
+        <v>145</v>
+      </c>
+      <c r="C22" t="s">
         <v>146</v>
-      </c>
-      <c r="C22" t="s">
-        <v>147</v>
       </c>
       <c r="D22">
         <v>88</v>
@@ -10007,29 +9996,29 @@
     </row>
     <row r="30" spans="2:6">
       <c r="B30" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="31" spans="2:6">
       <c r="C31" t="s">
+        <v>143</v>
+      </c>
+      <c r="D31" t="s">
         <v>144</v>
       </c>
-      <c r="D31" t="s">
-        <v>145</v>
-      </c>
       <c r="E31" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F31" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="32" spans="2:6">
       <c r="B32" t="s">
+        <v>145</v>
+      </c>
+      <c r="C32" t="s">
         <v>146</v>
-      </c>
-      <c r="C32" t="s">
-        <v>147</v>
       </c>
       <c r="D32">
         <v>88</v>

</xml_diff>

<commit_message>
feat: add production report logic, SQL query modules, and update build script to include new Excel templates.
</commit_message>
<xml_diff>
--- a/Eka_Report_back/MProductionReport.xlsx
+++ b/Eka_Report_back/MProductionReport.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\new\Eka_Report\Eka_Report_back\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD46AC6D-2A7E-4DD3-9340-A7AB58817560}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E8272D2-0639-4F16-95CC-5AE03D069A16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5760" yWindow="3540" windowWidth="17280" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Manag Report" sheetId="12" r:id="rId1"/>
@@ -5979,7 +5979,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -5994,73 +5994,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00B0F0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="-0.249977111117893"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -6433,7 +6367,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="125">
+  <cellXfs count="107">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -6466,19 +6400,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
@@ -6495,18 +6417,8 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -6514,90 +6426,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="11" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="12" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="14" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -6606,51 +6442,51 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="27" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="28" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="26" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="18" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="25" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
@@ -6658,37 +6494,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="16" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -6704,35 +6509,108 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="18" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="27" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="28" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="26" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7064,110 +6942,110 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21">
-      <c r="A1" s="76" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="77"/>
-      <c r="C1" s="77"/>
-      <c r="D1" s="77"/>
-      <c r="E1" s="77"/>
-      <c r="F1" s="77"/>
-      <c r="G1" s="77"/>
-      <c r="H1" s="77"/>
-      <c r="I1" s="77"/>
-      <c r="J1" s="77"/>
-      <c r="K1" s="77"/>
-      <c r="L1" s="77"/>
-      <c r="M1" s="77"/>
-      <c r="N1" s="77"/>
-      <c r="O1" s="77"/>
-      <c r="P1" s="77"/>
-      <c r="Q1" s="77"/>
-      <c r="R1" s="77"/>
-      <c r="S1" s="77"/>
-      <c r="T1" s="77"/>
-      <c r="U1" s="78"/>
+      <c r="A1" s="74" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="75"/>
+      <c r="C1" s="75"/>
+      <c r="D1" s="75"/>
+      <c r="E1" s="75"/>
+      <c r="F1" s="75"/>
+      <c r="G1" s="75"/>
+      <c r="H1" s="75"/>
+      <c r="I1" s="75"/>
+      <c r="J1" s="75"/>
+      <c r="K1" s="75"/>
+      <c r="L1" s="75"/>
+      <c r="M1" s="75"/>
+      <c r="N1" s="75"/>
+      <c r="O1" s="75"/>
+      <c r="P1" s="75"/>
+      <c r="Q1" s="75"/>
+      <c r="R1" s="75"/>
+      <c r="S1" s="75"/>
+      <c r="T1" s="75"/>
+      <c r="U1" s="76"/>
     </row>
     <row r="2" spans="1:21" ht="15" customHeight="1" thickBot="1">
-      <c r="A2" s="79"/>
-      <c r="B2" s="80"/>
-      <c r="C2" s="80"/>
-      <c r="D2" s="80"/>
-      <c r="E2" s="80"/>
-      <c r="F2" s="80"/>
-      <c r="G2" s="80"/>
-      <c r="H2" s="80"/>
-      <c r="I2" s="80"/>
-      <c r="J2" s="80"/>
-      <c r="K2" s="80"/>
-      <c r="L2" s="80"/>
-      <c r="M2" s="80"/>
-      <c r="N2" s="80"/>
-      <c r="O2" s="80"/>
-      <c r="P2" s="80"/>
-      <c r="Q2" s="80"/>
-      <c r="R2" s="80"/>
-      <c r="S2" s="80"/>
-      <c r="T2" s="80"/>
-      <c r="U2" s="81"/>
+      <c r="A2" s="77"/>
+      <c r="B2" s="78"/>
+      <c r="C2" s="78"/>
+      <c r="D2" s="78"/>
+      <c r="E2" s="78"/>
+      <c r="F2" s="78"/>
+      <c r="G2" s="78"/>
+      <c r="H2" s="78"/>
+      <c r="I2" s="78"/>
+      <c r="J2" s="78"/>
+      <c r="K2" s="78"/>
+      <c r="L2" s="78"/>
+      <c r="M2" s="78"/>
+      <c r="N2" s="78"/>
+      <c r="O2" s="78"/>
+      <c r="P2" s="78"/>
+      <c r="Q2" s="78"/>
+      <c r="R2" s="78"/>
+      <c r="S2" s="78"/>
+      <c r="T2" s="78"/>
+      <c r="U2" s="79"/>
     </row>
     <row r="3" spans="1:21">
       <c r="A3" s="3"/>
-      <c r="B3" s="56"/>
-      <c r="C3" s="56"/>
-      <c r="D3" s="56"/>
-      <c r="E3" s="56"/>
-      <c r="F3" s="56"/>
-      <c r="G3" s="56"/>
-      <c r="H3" s="56"/>
-      <c r="I3" s="56"/>
-      <c r="J3" s="56"/>
-      <c r="K3" s="56"/>
-      <c r="L3" s="56"/>
-      <c r="M3" s="56"/>
-      <c r="N3" s="56"/>
-      <c r="O3" s="56"/>
-      <c r="P3" s="56"/>
-      <c r="Q3" s="56"/>
-      <c r="R3" s="56"/>
-      <c r="S3" s="56"/>
-      <c r="T3" s="56"/>
+      <c r="B3" s="25"/>
+      <c r="C3" s="25"/>
+      <c r="D3" s="25"/>
+      <c r="E3" s="25"/>
+      <c r="F3" s="25"/>
+      <c r="G3" s="25"/>
+      <c r="H3" s="25"/>
+      <c r="I3" s="25"/>
+      <c r="J3" s="25"/>
+      <c r="K3" s="25"/>
+      <c r="L3" s="25"/>
+      <c r="M3" s="25"/>
+      <c r="N3" s="25"/>
+      <c r="O3" s="25"/>
+      <c r="P3" s="25"/>
+      <c r="Q3" s="25"/>
+      <c r="R3" s="25"/>
+      <c r="S3" s="25"/>
+      <c r="T3" s="25"/>
       <c r="U3" s="4"/>
     </row>
     <row r="4" spans="1:21" ht="15" customHeight="1">
-      <c r="A4" s="67" t="s">
+      <c r="A4" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="83" t="s">
+      <c r="B4" s="80" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="74"/>
-      <c r="P4" s="82" t="s">
+      <c r="C4" s="46"/>
+      <c r="P4" s="67" t="s">
         <v>1</v>
       </c>
-      <c r="Q4" s="73"/>
-      <c r="R4" s="73"/>
-      <c r="S4" s="73"/>
-      <c r="T4" s="74"/>
-      <c r="U4" s="35" t="s">
+      <c r="Q4" s="45"/>
+      <c r="R4" s="45"/>
+      <c r="S4" s="45"/>
+      <c r="T4" s="46"/>
+      <c r="U4" s="24" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:21" ht="15" customHeight="1">
-      <c r="A5" s="67" t="s">
+      <c r="A5" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="75">
+      <c r="B5" s="73">
         <v>0.69398981410879634</v>
       </c>
-      <c r="C5" s="74"/>
+      <c r="C5" s="46"/>
       <c r="P5" s="72" t="s">
         <v>3</v>
       </c>
-      <c r="Q5" s="73"/>
-      <c r="R5" s="73"/>
-      <c r="S5" s="73"/>
-      <c r="T5" s="74"/>
+      <c r="Q5" s="45"/>
+      <c r="R5" s="45"/>
+      <c r="S5" s="45"/>
+      <c r="T5" s="46"/>
       <c r="U5" s="6">
         <f>Daily!L3</f>
         <v>0</v>
@@ -7178,10 +7056,10 @@
       <c r="P6" s="72" t="s">
         <v>6</v>
       </c>
-      <c r="Q6" s="73"/>
-      <c r="R6" s="73"/>
-      <c r="S6" s="73"/>
-      <c r="T6" s="74"/>
+      <c r="Q6" s="45"/>
+      <c r="R6" s="45"/>
+      <c r="S6" s="45"/>
+      <c r="T6" s="46"/>
       <c r="U6" s="6">
         <f>Daily!M3</f>
         <v>0</v>
@@ -7189,39 +7067,39 @@
     </row>
     <row r="7" spans="1:21">
       <c r="A7" s="5"/>
-      <c r="S7" s="66"/>
-      <c r="T7" s="66"/>
+      <c r="S7" s="32"/>
+      <c r="T7" s="32"/>
       <c r="U7" s="7"/>
     </row>
     <row r="8" spans="1:21">
-      <c r="A8" s="84"/>
-      <c r="B8" s="85"/>
-      <c r="C8" s="85"/>
-      <c r="D8" s="86"/>
-      <c r="E8" s="82" t="s">
+      <c r="A8" s="44"/>
+      <c r="B8" s="53"/>
+      <c r="C8" s="53"/>
+      <c r="D8" s="54"/>
+      <c r="E8" s="67" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="73"/>
-      <c r="G8" s="74"/>
-      <c r="H8" s="59"/>
-      <c r="I8" s="82" t="s">
+      <c r="F8" s="45"/>
+      <c r="G8" s="46"/>
+      <c r="H8" s="26"/>
+      <c r="I8" s="67" t="s">
         <v>9</v>
       </c>
-      <c r="J8" s="73"/>
-      <c r="K8" s="73"/>
-      <c r="L8" s="73"/>
-      <c r="M8" s="74"/>
-      <c r="N8" s="82" t="s">
+      <c r="J8" s="45"/>
+      <c r="K8" s="45"/>
+      <c r="L8" s="45"/>
+      <c r="M8" s="46"/>
+      <c r="N8" s="67" t="s">
         <v>10</v>
       </c>
-      <c r="O8" s="73"/>
-      <c r="P8" s="74"/>
-      <c r="Q8" s="82" t="s">
+      <c r="O8" s="45"/>
+      <c r="P8" s="46"/>
+      <c r="Q8" s="67" t="s">
         <v>11</v>
       </c>
-      <c r="R8" s="73"/>
-      <c r="S8" s="74"/>
-      <c r="T8" s="30" t="s">
+      <c r="R8" s="45"/>
+      <c r="S8" s="46"/>
+      <c r="T8" s="22" t="s">
         <v>12</v>
       </c>
       <c r="U8" s="9" t="s">
@@ -7229,34 +7107,34 @@
       </c>
     </row>
     <row r="9" spans="1:21">
-      <c r="A9" s="87"/>
-      <c r="B9" s="88"/>
-      <c r="C9" s="88"/>
-      <c r="D9" s="89"/>
-      <c r="E9" s="90" t="s">
+      <c r="A9" s="55"/>
+      <c r="B9" s="56"/>
+      <c r="C9" s="56"/>
+      <c r="D9" s="57"/>
+      <c r="E9" s="70" t="s">
         <v>2</v>
       </c>
-      <c r="F9" s="73"/>
-      <c r="G9" s="74"/>
-      <c r="H9" s="59"/>
-      <c r="I9" s="82" t="s">
+      <c r="F9" s="45"/>
+      <c r="G9" s="46"/>
+      <c r="H9" s="26"/>
+      <c r="I9" s="67" t="s">
         <v>14</v>
       </c>
-      <c r="J9" s="73"/>
-      <c r="K9" s="73"/>
-      <c r="L9" s="73"/>
-      <c r="M9" s="74"/>
-      <c r="N9" s="90" t="s">
+      <c r="J9" s="45"/>
+      <c r="K9" s="45"/>
+      <c r="L9" s="45"/>
+      <c r="M9" s="46"/>
+      <c r="N9" s="70" t="s">
         <v>15</v>
       </c>
-      <c r="O9" s="73"/>
-      <c r="P9" s="74"/>
-      <c r="Q9" s="90" t="s">
+      <c r="O9" s="45"/>
+      <c r="P9" s="46"/>
+      <c r="Q9" s="70" t="s">
         <v>16</v>
       </c>
-      <c r="R9" s="73"/>
-      <c r="S9" s="74"/>
-      <c r="T9" s="30">
+      <c r="R9" s="45"/>
+      <c r="S9" s="46"/>
+      <c r="T9" s="22">
         <f>YTD!C12</f>
         <v>0</v>
       </c>
@@ -7266,56 +7144,56 @@
       </c>
     </row>
     <row r="10" spans="1:21">
-      <c r="A10" s="91" t="s">
+      <c r="A10" s="52" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="73"/>
-      <c r="C10" s="73"/>
-      <c r="D10" s="74"/>
-      <c r="E10" s="59" t="s">
+      <c r="B10" s="45"/>
+      <c r="C10" s="45"/>
+      <c r="D10" s="46"/>
+      <c r="E10" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="F10" s="59" t="s">
+      <c r="F10" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="G10" s="59" t="s">
+      <c r="G10" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="H10" s="59"/>
-      <c r="I10" s="59" t="s">
+      <c r="H10" s="26"/>
+      <c r="I10" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="J10" s="59" t="s">
+      <c r="J10" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="K10" s="59" t="s">
+      <c r="K10" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="L10" s="59" t="s">
+      <c r="L10" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="M10" s="59" t="s">
+      <c r="M10" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="N10" s="59" t="s">
+      <c r="N10" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="O10" s="59" t="s">
+      <c r="O10" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="P10" s="59" t="s">
+      <c r="P10" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="Q10" s="59" t="s">
+      <c r="Q10" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="R10" s="59" t="s">
+      <c r="R10" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="S10" s="59" t="s">
+      <c r="S10" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="T10" s="59" t="s">
+      <c r="T10" s="26" t="s">
         <v>19</v>
       </c>
       <c r="U10" s="10" t="s">
@@ -7323,290 +7201,290 @@
       </c>
     </row>
     <row r="11" spans="1:21">
-      <c r="A11" s="92" t="s">
+      <c r="A11" s="103" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="73"/>
-      <c r="C11" s="73"/>
-      <c r="D11" s="74"/>
-      <c r="E11" s="64">
+      <c r="B11" s="48"/>
+      <c r="C11" s="48"/>
+      <c r="D11" s="49"/>
+      <c r="E11" s="30">
         <v>70</v>
       </c>
-      <c r="F11" s="44">
+      <c r="F11" s="30">
         <v>23</v>
       </c>
-      <c r="G11" s="36">
+      <c r="G11" s="30">
         <v>-47</v>
       </c>
-      <c r="H11" s="63"/>
-      <c r="I11" s="36">
+      <c r="H11" s="31"/>
+      <c r="I11" s="30">
         <v>15</v>
       </c>
-      <c r="J11" s="36">
+      <c r="J11" s="30">
         <v>8</v>
       </c>
-      <c r="K11" s="36">
-        <v>0</v>
-      </c>
-      <c r="L11" s="36">
-        <v>0</v>
-      </c>
-      <c r="M11" s="36">
-        <v>0</v>
-      </c>
-      <c r="N11" s="37">
+      <c r="K11" s="30">
+        <v>0</v>
+      </c>
+      <c r="L11" s="30">
+        <v>0</v>
+      </c>
+      <c r="M11" s="30">
+        <v>0</v>
+      </c>
+      <c r="N11" s="30">
         <v>10</v>
       </c>
-      <c r="O11" s="52">
+      <c r="O11" s="30">
         <v>2</v>
       </c>
-      <c r="P11" s="36">
+      <c r="P11" s="30">
         <v>-8</v>
       </c>
-      <c r="Q11" s="36">
+      <c r="Q11" s="30">
         <v>70</v>
       </c>
-      <c r="R11" s="48">
+      <c r="R11" s="30">
         <v>23</v>
       </c>
-      <c r="S11" s="36">
+      <c r="S11" s="30">
         <v>-47</v>
       </c>
-      <c r="T11" s="36">
+      <c r="T11" s="30">
         <v>288</v>
       </c>
-      <c r="U11" s="38">
+      <c r="U11" s="104">
         <v>68</v>
       </c>
     </row>
     <row r="12" spans="1:21">
-      <c r="A12" s="93" t="s">
+      <c r="A12" s="103" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="73"/>
-      <c r="C12" s="73"/>
-      <c r="D12" s="74"/>
-      <c r="E12" s="64">
+      <c r="B12" s="48"/>
+      <c r="C12" s="48"/>
+      <c r="D12" s="49"/>
+      <c r="E12" s="30">
         <v>80</v>
       </c>
-      <c r="F12" s="46">
+      <c r="F12" s="30">
         <v>29</v>
       </c>
-      <c r="G12" s="36">
+      <c r="G12" s="30">
         <v>-51</v>
       </c>
-      <c r="H12" s="63"/>
-      <c r="I12" s="36">
+      <c r="H12" s="31"/>
+      <c r="I12" s="30">
         <v>24</v>
       </c>
-      <c r="J12" s="36">
+      <c r="J12" s="30">
         <v>5</v>
       </c>
-      <c r="K12" s="36">
-        <v>0</v>
-      </c>
-      <c r="L12" s="36">
-        <v>0</v>
-      </c>
-      <c r="M12" s="36">
-        <v>0</v>
-      </c>
-      <c r="N12" s="37">
+      <c r="K12" s="30">
+        <v>0</v>
+      </c>
+      <c r="L12" s="30">
+        <v>0</v>
+      </c>
+      <c r="M12" s="30">
+        <v>0</v>
+      </c>
+      <c r="N12" s="30">
         <v>10</v>
       </c>
-      <c r="O12" s="54">
+      <c r="O12" s="30">
         <v>1</v>
       </c>
-      <c r="P12" s="36">
+      <c r="P12" s="30">
         <v>-9</v>
       </c>
-      <c r="Q12" s="36">
+      <c r="Q12" s="30">
         <v>80</v>
       </c>
-      <c r="R12" s="50">
+      <c r="R12" s="30">
         <v>29</v>
       </c>
-      <c r="S12" s="36">
+      <c r="S12" s="30">
         <v>-51</v>
       </c>
-      <c r="T12" s="36">
+      <c r="T12" s="30">
         <v>366</v>
       </c>
-      <c r="U12" s="38">
+      <c r="U12" s="104">
         <v>68</v>
       </c>
     </row>
     <row r="13" spans="1:21">
-      <c r="A13" s="93" t="s">
+      <c r="A13" s="103" t="s">
         <v>28</v>
       </c>
-      <c r="B13" s="73"/>
-      <c r="C13" s="73"/>
-      <c r="D13" s="74"/>
-      <c r="E13" s="65">
+      <c r="B13" s="48"/>
+      <c r="C13" s="48"/>
+      <c r="D13" s="49"/>
+      <c r="E13" s="31">
         <f>Monthly!D4</f>
         <v>0</v>
       </c>
-      <c r="F13" s="65">
+      <c r="F13" s="31">
         <f>Monthly!E4</f>
         <v>0</v>
       </c>
-      <c r="G13" s="63">
+      <c r="G13" s="31">
         <f>Monthly!F4</f>
         <v>0</v>
       </c>
-      <c r="H13" s="32"/>
-      <c r="I13" s="63">
+      <c r="H13" s="105"/>
+      <c r="I13" s="31">
         <f>Weely!E4</f>
         <v>0</v>
       </c>
-      <c r="J13" s="63">
+      <c r="J13" s="31">
         <f>Weely!G4</f>
         <v>0</v>
       </c>
-      <c r="K13" s="63">
+      <c r="K13" s="31">
         <f>Weely!I4</f>
         <v>0</v>
       </c>
-      <c r="L13" s="63">
+      <c r="L13" s="31">
         <f>Weely!K4</f>
         <v>0</v>
       </c>
-      <c r="M13" s="63">
+      <c r="M13" s="31">
         <f>Weely!M4</f>
         <v>0</v>
       </c>
-      <c r="N13" s="27">
+      <c r="N13" s="31">
         <f>Daily!D4</f>
         <v>0</v>
       </c>
-      <c r="O13" s="27">
+      <c r="O13" s="31">
         <f>Daily!E4</f>
         <v>0</v>
       </c>
-      <c r="P13" s="63">
+      <c r="P13" s="31">
         <f>Daily!F4</f>
         <v>0</v>
       </c>
-      <c r="Q13" s="63">
+      <c r="Q13" s="31">
         <f>MTD!D4</f>
         <v>0</v>
       </c>
-      <c r="R13" s="63">
+      <c r="R13" s="31">
         <f>MTD!E4</f>
         <v>0</v>
       </c>
-      <c r="S13" s="63">
+      <c r="S13" s="31">
         <f>MTD!F4</f>
         <v>0</v>
       </c>
-      <c r="T13" s="63">
+      <c r="T13" s="31">
         <f>YTD!E4</f>
         <v>0</v>
       </c>
-      <c r="U13" s="6">
+      <c r="U13" s="106">
         <f>PrevFY!E4</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:21">
-      <c r="A14" s="93" t="s">
+      <c r="A14" s="103" t="s">
         <v>29</v>
       </c>
-      <c r="B14" s="73"/>
-      <c r="C14" s="73"/>
-      <c r="D14" s="74"/>
-      <c r="E14" s="65">
+      <c r="B14" s="48"/>
+      <c r="C14" s="48"/>
+      <c r="D14" s="49"/>
+      <c r="E14" s="31">
         <f>Monthly!D5</f>
         <v>0</v>
       </c>
-      <c r="F14" s="65">
+      <c r="F14" s="31">
         <f>Monthly!E5</f>
         <v>0</v>
       </c>
-      <c r="G14" s="63">
+      <c r="G14" s="31">
         <f>Monthly!F5</f>
         <v>0</v>
       </c>
-      <c r="H14" s="32"/>
-      <c r="I14" s="63">
+      <c r="H14" s="105"/>
+      <c r="I14" s="31">
         <f>Weely!E5</f>
         <v>0</v>
       </c>
-      <c r="J14" s="63">
+      <c r="J14" s="31">
         <f>Weely!G5</f>
         <v>0</v>
       </c>
-      <c r="K14" s="63">
+      <c r="K14" s="31">
         <f>Weely!I5</f>
         <v>0</v>
       </c>
-      <c r="L14" s="63">
+      <c r="L14" s="31">
         <f>Weely!K5</f>
         <v>0</v>
       </c>
-      <c r="M14" s="63">
+      <c r="M14" s="31">
         <f>Weely!M5</f>
         <v>0</v>
       </c>
-      <c r="N14" s="27">
+      <c r="N14" s="31">
         <f>Daily!D5</f>
         <v>0</v>
       </c>
-      <c r="O14" s="27">
+      <c r="O14" s="31">
         <f>Daily!E5</f>
         <v>0</v>
       </c>
-      <c r="P14" s="63">
+      <c r="P14" s="31">
         <f>Daily!F5</f>
         <v>0</v>
       </c>
-      <c r="Q14" s="63">
+      <c r="Q14" s="31">
         <f>MTD!D5</f>
         <v>0</v>
       </c>
-      <c r="R14" s="63">
+      <c r="R14" s="31">
         <f>MTD!E5</f>
         <v>0</v>
       </c>
-      <c r="S14" s="63">
+      <c r="S14" s="31">
         <f>MTD!F5</f>
         <v>0</v>
       </c>
-      <c r="T14" s="63">
+      <c r="T14" s="31">
         <f>YTD!E5</f>
         <v>0</v>
       </c>
-      <c r="U14" s="6">
+      <c r="U14" s="106">
         <f>PrevFY!E5</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:21">
-      <c r="A15" s="84"/>
-      <c r="B15" s="74"/>
-      <c r="C15" s="90" t="s">
+      <c r="A15" s="44"/>
+      <c r="B15" s="46"/>
+      <c r="C15" s="70" t="s">
         <v>30</v>
       </c>
-      <c r="D15" s="74"/>
-      <c r="E15" s="90" t="s">
+      <c r="D15" s="46"/>
+      <c r="E15" s="70" t="s">
         <v>2</v>
       </c>
-      <c r="F15" s="73"/>
-      <c r="G15" s="73"/>
-      <c r="H15" s="74"/>
-      <c r="I15" s="82" t="s">
+      <c r="F15" s="45"/>
+      <c r="G15" s="45"/>
+      <c r="H15" s="46"/>
+      <c r="I15" s="67" t="s">
         <v>31</v>
       </c>
-      <c r="J15" s="73"/>
-      <c r="K15" s="73"/>
-      <c r="L15" s="73"/>
-      <c r="M15" s="74"/>
-      <c r="N15" s="90" t="s">
+      <c r="J15" s="45"/>
+      <c r="K15" s="45"/>
+      <c r="L15" s="45"/>
+      <c r="M15" s="46"/>
+      <c r="N15" s="70" t="s">
         <v>15</v>
       </c>
-      <c r="O15" s="73"/>
-      <c r="P15" s="74"/>
+      <c r="O15" s="45"/>
+      <c r="P15" s="46"/>
       <c r="Q15" s="11"/>
       <c r="R15" s="12"/>
       <c r="S15" s="12"/>
@@ -7614,170 +7492,170 @@
       <c r="U15" s="13"/>
     </row>
     <row r="16" spans="1:21">
-      <c r="A16" s="94"/>
-      <c r="B16" s="74"/>
-      <c r="C16" s="33" t="s">
+      <c r="A16" s="91"/>
+      <c r="B16" s="49"/>
+      <c r="C16" s="87" t="s">
         <v>32</v>
       </c>
-      <c r="D16" s="59" t="s">
+      <c r="D16" s="87" t="s">
         <v>33</v>
       </c>
-      <c r="E16" s="33" t="s">
+      <c r="E16" s="87" t="s">
         <v>32</v>
       </c>
-      <c r="F16" s="59" t="s">
+      <c r="F16" s="87" t="s">
         <v>33</v>
       </c>
-      <c r="G16" s="34" t="s">
+      <c r="G16" s="82" t="s">
         <v>34</v>
       </c>
-      <c r="H16" s="14" t="s">
+      <c r="H16" s="82" t="s">
         <v>35</v>
       </c>
-      <c r="I16" s="59" t="s">
+      <c r="I16" s="87" t="s">
         <v>21</v>
       </c>
-      <c r="J16" s="59" t="s">
+      <c r="J16" s="87" t="s">
         <v>22</v>
       </c>
-      <c r="K16" s="59" t="s">
+      <c r="K16" s="87" t="s">
         <v>23</v>
       </c>
-      <c r="L16" s="59" t="s">
+      <c r="L16" s="87" t="s">
         <v>24</v>
       </c>
-      <c r="M16" s="59" t="s">
+      <c r="M16" s="87" t="s">
         <v>25</v>
       </c>
-      <c r="N16" s="59" t="s">
+      <c r="N16" s="87" t="s">
         <v>36</v>
       </c>
-      <c r="O16" s="59" t="s">
+      <c r="O16" s="87" t="s">
         <v>33</v>
       </c>
-      <c r="P16" s="59" t="s">
+      <c r="P16" s="87" t="s">
         <v>37</v>
       </c>
-      <c r="Q16" s="15"/>
+      <c r="Q16" s="14"/>
       <c r="R16" s="1"/>
       <c r="S16" s="1"/>
       <c r="T16" s="1"/>
       <c r="U16" s="13"/>
     </row>
     <row r="17" spans="1:21">
-      <c r="A17" s="16" t="s">
+      <c r="A17" s="92" t="s">
         <v>38</v>
       </c>
-      <c r="B17" s="17" t="s">
+      <c r="B17" s="93" t="s">
         <v>39</v>
       </c>
-      <c r="C17" s="39">
+      <c r="C17" s="94">
         <v>68</v>
       </c>
-      <c r="D17" s="39">
+      <c r="D17" s="94">
         <v>68</v>
       </c>
-      <c r="E17" s="45">
+      <c r="E17" s="31">
         <f>Monthly!E12</f>
         <v>0</v>
       </c>
-      <c r="F17" s="47">
+      <c r="F17" s="31">
         <f>Monthly!E3</f>
         <v>0</v>
       </c>
-      <c r="G17" s="49">
+      <c r="G17" s="31">
         <f>YTD!E12</f>
         <v>0</v>
       </c>
-      <c r="H17" s="51">
+      <c r="H17" s="31">
         <f>YTD!E3</f>
         <v>0</v>
       </c>
-      <c r="I17" s="63">
+      <c r="I17" s="31">
         <f>Weely!E12</f>
         <v>0</v>
       </c>
-      <c r="J17" s="51">
+      <c r="J17" s="31">
         <f>Weely!G12</f>
         <v>0</v>
       </c>
-      <c r="K17" s="63">
+      <c r="K17" s="31">
         <f>Weely!I12</f>
         <v>0</v>
       </c>
-      <c r="L17" s="63">
+      <c r="L17" s="31">
         <f>Weely!K12</f>
         <v>0</v>
       </c>
-      <c r="M17" s="63">
+      <c r="M17" s="31">
         <f>Weely!M12</f>
         <v>0</v>
       </c>
-      <c r="N17" s="53">
+      <c r="N17" s="31">
         <f>Daily!E13</f>
         <v>0</v>
       </c>
-      <c r="O17" s="55">
+      <c r="O17" s="31">
         <f>Daily!E3</f>
         <v>0</v>
       </c>
-      <c r="P17" s="63">
+      <c r="P17" s="31">
         <f>SUM(N17:O17)</f>
         <v>0</v>
       </c>
-      <c r="Q17" s="15"/>
+      <c r="Q17" s="14"/>
       <c r="R17" s="1"/>
       <c r="S17" s="1"/>
       <c r="T17" s="1"/>
       <c r="U17" s="13"/>
     </row>
     <row r="18" spans="1:21">
-      <c r="A18" s="18" t="s">
+      <c r="A18" s="95" t="s">
         <v>40</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="93" t="s">
         <v>39</v>
       </c>
-      <c r="C18" s="36">
+      <c r="C18" s="30">
         <v>68</v>
       </c>
-      <c r="D18" s="36">
+      <c r="D18" s="30">
         <v>68</v>
       </c>
-      <c r="E18" s="36">
+      <c r="E18" s="30">
         <v>4</v>
       </c>
-      <c r="F18" s="36">
+      <c r="F18" s="30">
         <v>4</v>
       </c>
-      <c r="G18" s="36">
+      <c r="G18" s="30">
         <v>4</v>
       </c>
-      <c r="H18" s="36">
+      <c r="H18" s="30">
         <v>4</v>
       </c>
-      <c r="I18" s="36">
-        <v>0</v>
-      </c>
-      <c r="J18" s="36" t="s">
+      <c r="I18" s="30">
+        <v>0</v>
+      </c>
+      <c r="J18" s="30" t="s">
         <v>150</v>
       </c>
-      <c r="K18" s="36">
-        <v>0</v>
-      </c>
-      <c r="L18" s="36">
-        <v>0</v>
-      </c>
-      <c r="M18" s="36">
-        <v>0</v>
-      </c>
-      <c r="N18" s="37" t="s">
+      <c r="K18" s="30">
+        <v>0</v>
+      </c>
+      <c r="L18" s="30">
+        <v>0</v>
+      </c>
+      <c r="M18" s="30">
+        <v>0</v>
+      </c>
+      <c r="N18" s="30" t="s">
         <v>150</v>
       </c>
-      <c r="O18" s="37" t="s">
+      <c r="O18" s="30" t="s">
         <v>150</v>
       </c>
-      <c r="P18" s="63">
+      <c r="P18" s="31">
         <f>SUM(N18:O18)</f>
         <v>0</v>
       </c>
@@ -7788,286 +7666,322 @@
       <c r="U18" s="13"/>
     </row>
     <row r="19" spans="1:21">
-      <c r="A19" s="31"/>
-      <c r="B19" s="8"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
-      <c r="H19" s="8"/>
-      <c r="I19" s="82" t="s">
+      <c r="A19" s="96"/>
+      <c r="B19" s="97"/>
+      <c r="C19" s="97"/>
+      <c r="D19" s="97"/>
+      <c r="E19" s="97"/>
+      <c r="F19" s="97"/>
+      <c r="G19" s="97"/>
+      <c r="H19" s="97"/>
+      <c r="I19" s="83" t="s">
         <v>41</v>
       </c>
-      <c r="J19" s="73"/>
-      <c r="K19" s="73"/>
-      <c r="L19" s="73"/>
-      <c r="M19" s="74"/>
-      <c r="N19" s="8"/>
-      <c r="O19" s="8"/>
-      <c r="P19" s="8"/>
+      <c r="J19" s="48"/>
+      <c r="K19" s="48"/>
+      <c r="L19" s="48"/>
+      <c r="M19" s="49"/>
+      <c r="N19" s="97"/>
+      <c r="O19" s="97"/>
+      <c r="P19" s="97"/>
       <c r="Q19" s="8"/>
       <c r="R19" s="8"/>
       <c r="S19" s="8"/>
       <c r="T19" s="8"/>
-      <c r="U19" s="19"/>
+      <c r="U19" s="15"/>
     </row>
     <row r="20" spans="1:21">
-      <c r="A20" s="5"/>
-      <c r="I20" s="59" t="s">
+      <c r="A20" s="98"/>
+      <c r="B20" s="99"/>
+      <c r="C20" s="99"/>
+      <c r="D20" s="99"/>
+      <c r="E20" s="99"/>
+      <c r="F20" s="99"/>
+      <c r="G20" s="99"/>
+      <c r="H20" s="99"/>
+      <c r="I20" s="87" t="s">
         <v>21</v>
       </c>
-      <c r="J20" s="59" t="s">
+      <c r="J20" s="87" t="s">
         <v>22</v>
       </c>
-      <c r="K20" s="59" t="s">
+      <c r="K20" s="87" t="s">
         <v>23</v>
       </c>
-      <c r="L20" s="59" t="s">
+      <c r="L20" s="87" t="s">
         <v>24</v>
       </c>
-      <c r="M20" s="59" t="s">
+      <c r="M20" s="87" t="s">
         <v>25</v>
       </c>
+      <c r="N20" s="99"/>
+      <c r="O20" s="99"/>
+      <c r="P20" s="99"/>
       <c r="U20" s="7"/>
     </row>
     <row r="21" spans="1:21">
-      <c r="A21" s="5"/>
-      <c r="I21" s="36">
-        <v>0</v>
-      </c>
-      <c r="J21" s="36" t="s">
+      <c r="A21" s="98"/>
+      <c r="B21" s="99"/>
+      <c r="C21" s="99"/>
+      <c r="D21" s="99"/>
+      <c r="E21" s="99"/>
+      <c r="F21" s="99"/>
+      <c r="G21" s="99"/>
+      <c r="H21" s="99"/>
+      <c r="I21" s="30">
+        <v>0</v>
+      </c>
+      <c r="J21" s="30" t="s">
         <v>150</v>
       </c>
-      <c r="K21" s="36">
-        <v>0</v>
-      </c>
-      <c r="L21" s="36">
-        <v>0</v>
-      </c>
-      <c r="M21" s="36">
-        <v>0</v>
-      </c>
+      <c r="K21" s="30">
+        <v>0</v>
+      </c>
+      <c r="L21" s="30">
+        <v>0</v>
+      </c>
+      <c r="M21" s="30">
+        <v>0</v>
+      </c>
+      <c r="N21" s="99"/>
+      <c r="O21" s="99"/>
+      <c r="P21" s="99"/>
       <c r="U21" s="7"/>
     </row>
     <row r="22" spans="1:21">
-      <c r="A22" s="5"/>
-      <c r="H22" s="20" t="s">
+      <c r="A22" s="98"/>
+      <c r="B22" s="99"/>
+      <c r="C22" s="99"/>
+      <c r="D22" s="99"/>
+      <c r="E22" s="99"/>
+      <c r="F22" s="99"/>
+      <c r="G22" s="99"/>
+      <c r="H22" s="100" t="s">
         <v>39</v>
       </c>
-      <c r="I22" s="36">
-        <v>0</v>
-      </c>
-      <c r="J22" s="36" t="s">
+      <c r="I22" s="30">
+        <v>0</v>
+      </c>
+      <c r="J22" s="30" t="s">
         <v>150</v>
       </c>
-      <c r="K22" s="36">
-        <v>0</v>
-      </c>
-      <c r="L22" s="36">
-        <v>0</v>
-      </c>
-      <c r="M22" s="36">
-        <v>0</v>
-      </c>
+      <c r="K22" s="30">
+        <v>0</v>
+      </c>
+      <c r="L22" s="30">
+        <v>0</v>
+      </c>
+      <c r="M22" s="30">
+        <v>0</v>
+      </c>
+      <c r="N22" s="99"/>
+      <c r="O22" s="99"/>
+      <c r="P22" s="99"/>
       <c r="U22" s="7"/>
     </row>
     <row r="23" spans="1:21">
-      <c r="A23" s="5"/>
-      <c r="I23" s="82" t="s">
+      <c r="A23" s="98"/>
+      <c r="B23" s="99"/>
+      <c r="C23" s="99"/>
+      <c r="D23" s="99"/>
+      <c r="E23" s="99"/>
+      <c r="F23" s="99"/>
+      <c r="G23" s="99"/>
+      <c r="H23" s="99"/>
+      <c r="I23" s="83" t="s">
         <v>42</v>
       </c>
-      <c r="J23" s="73"/>
-      <c r="K23" s="73"/>
-      <c r="L23" s="73"/>
-      <c r="M23" s="74"/>
-      <c r="N23" s="100" t="s">
+      <c r="J23" s="48"/>
+      <c r="K23" s="48"/>
+      <c r="L23" s="48"/>
+      <c r="M23" s="49"/>
+      <c r="N23" s="101" t="s">
         <v>15</v>
       </c>
-      <c r="O23" s="73"/>
-      <c r="P23" s="74"/>
+      <c r="O23" s="48"/>
+      <c r="P23" s="49"/>
       <c r="U23" s="7"/>
     </row>
     <row r="24" spans="1:21">
-      <c r="A24" s="94"/>
-      <c r="B24" s="74"/>
-      <c r="C24" s="59" t="s">
+      <c r="A24" s="91"/>
+      <c r="B24" s="49"/>
+      <c r="C24" s="87" t="s">
         <v>28</v>
       </c>
-      <c r="D24" s="59" t="s">
+      <c r="D24" s="87" t="s">
         <v>29</v>
       </c>
-      <c r="E24" s="59" t="s">
+      <c r="E24" s="87" t="s">
         <v>28</v>
       </c>
-      <c r="F24" s="59" t="s">
+      <c r="F24" s="87" t="s">
         <v>29</v>
       </c>
-      <c r="G24" s="59" t="s">
+      <c r="G24" s="87" t="s">
         <v>43</v>
       </c>
-      <c r="H24" s="59" t="s">
+      <c r="H24" s="87" t="s">
         <v>44</v>
       </c>
-      <c r="I24" s="59" t="s">
+      <c r="I24" s="87" t="s">
         <v>21</v>
       </c>
-      <c r="J24" s="59" t="s">
+      <c r="J24" s="87" t="s">
         <v>22</v>
       </c>
-      <c r="K24" s="59" t="s">
+      <c r="K24" s="87" t="s">
         <v>23</v>
       </c>
-      <c r="L24" s="59" t="s">
+      <c r="L24" s="87" t="s">
         <v>24</v>
       </c>
-      <c r="M24" s="59" t="s">
+      <c r="M24" s="87" t="s">
         <v>25</v>
       </c>
-      <c r="N24" s="59" t="s">
+      <c r="N24" s="87" t="s">
         <v>28</v>
       </c>
-      <c r="O24" s="59" t="s">
+      <c r="O24" s="87" t="s">
         <v>29</v>
       </c>
-      <c r="P24" s="59" t="s">
+      <c r="P24" s="87" t="s">
         <v>37</v>
       </c>
-      <c r="Q24" s="15"/>
+      <c r="Q24" s="14"/>
       <c r="R24" s="1"/>
       <c r="S24" s="1"/>
       <c r="T24" s="1"/>
       <c r="U24" s="13"/>
     </row>
     <row r="25" spans="1:21">
-      <c r="A25" s="16" t="s">
+      <c r="A25" s="92" t="s">
         <v>38</v>
       </c>
-      <c r="B25" s="17" t="s">
+      <c r="B25" s="93" t="s">
         <v>39</v>
       </c>
-      <c r="C25" s="26">
+      <c r="C25" s="102">
         <f>PrevFY!E18</f>
         <v>0</v>
       </c>
-      <c r="D25" s="26">
+      <c r="D25" s="102">
         <f>PrevFY!E9</f>
         <v>0</v>
       </c>
-      <c r="E25" s="63">
+      <c r="E25" s="31">
         <f>Monthly!E18</f>
         <v>0</v>
       </c>
-      <c r="F25" s="63">
+      <c r="F25" s="31">
         <f>Monthly!E9</f>
         <v>0</v>
       </c>
-      <c r="G25" s="63">
+      <c r="G25" s="31">
         <f>YTD!E18</f>
         <v>0</v>
       </c>
-      <c r="H25" s="63">
+      <c r="H25" s="31">
         <f>YTD!E9</f>
         <v>0</v>
       </c>
-      <c r="I25" s="63">
+      <c r="I25" s="31">
         <f>Weely!E18</f>
         <v>0</v>
       </c>
-      <c r="J25" s="63">
+      <c r="J25" s="31">
         <f>Weely!G18</f>
         <v>0</v>
       </c>
-      <c r="K25" s="63">
+      <c r="K25" s="31">
         <f>Weely!I18</f>
         <v>0</v>
       </c>
-      <c r="L25" s="63">
+      <c r="L25" s="31">
         <f>Weely!K18</f>
         <v>0</v>
       </c>
-      <c r="M25" s="63">
+      <c r="M25" s="31">
         <f>Weely!M18</f>
         <v>0</v>
       </c>
-      <c r="N25" s="63">
+      <c r="N25" s="31">
         <f>Daily!E19</f>
         <v>0</v>
       </c>
-      <c r="O25" s="63">
+      <c r="O25" s="31">
         <f>Daily!E9</f>
         <v>0</v>
       </c>
-      <c r="P25" s="63">
+      <c r="P25" s="31">
         <f>SUM(N25:O25)</f>
         <v>0</v>
       </c>
-      <c r="Q25" s="15"/>
+      <c r="Q25" s="14"/>
       <c r="R25" s="1"/>
       <c r="S25" s="1"/>
       <c r="T25" s="1"/>
       <c r="U25" s="13"/>
     </row>
     <row r="26" spans="1:21">
-      <c r="A26" s="18" t="s">
+      <c r="A26" s="95" t="s">
         <v>40</v>
       </c>
-      <c r="B26" s="17" t="s">
+      <c r="B26" s="93" t="s">
         <v>39</v>
       </c>
-      <c r="C26" s="63">
+      <c r="C26" s="31">
         <f>PrevFY!E38</f>
         <v>0</v>
       </c>
-      <c r="D26" s="63">
+      <c r="D26" s="31">
         <f>PrevFY!E28</f>
         <v>0</v>
       </c>
-      <c r="E26" s="63">
+      <c r="E26" s="31">
         <f>Monthly!E38</f>
         <v>0</v>
       </c>
-      <c r="F26" s="63">
+      <c r="F26" s="31">
         <f>Monthly!E28</f>
         <v>0</v>
       </c>
-      <c r="G26" s="63">
+      <c r="G26" s="31">
         <f>YTD!E38</f>
         <v>0</v>
       </c>
-      <c r="H26" s="63">
+      <c r="H26" s="31">
         <f>YTD!E28</f>
         <v>0</v>
       </c>
-      <c r="I26" s="63">
+      <c r="I26" s="31">
         <f>Weely!E38</f>
         <v>0</v>
       </c>
-      <c r="J26" s="63">
+      <c r="J26" s="31">
         <f>Weely!G38</f>
         <v>0</v>
       </c>
-      <c r="K26" s="63">
+      <c r="K26" s="31">
         <f>Weely!I38</f>
         <v>0</v>
       </c>
-      <c r="L26" s="63">
+      <c r="L26" s="31">
         <f>Weely!K38</f>
         <v>0</v>
       </c>
-      <c r="M26" s="63">
+      <c r="M26" s="31">
         <f>Weely!M38</f>
         <v>0</v>
       </c>
-      <c r="N26" s="27">
+      <c r="N26" s="31">
         <f>Daily!E38</f>
         <v>0</v>
       </c>
-      <c r="O26" s="27">
+      <c r="O26" s="31">
         <f>Daily!E28</f>
         <v>0</v>
       </c>
-      <c r="P26" s="63">
+      <c r="P26" s="31">
         <f>SUM(N26:O26)</f>
         <v>0</v>
       </c>
@@ -8078,7 +7992,7 @@
       <c r="U26" s="13"/>
     </row>
     <row r="27" spans="1:21">
-      <c r="A27" s="31"/>
+      <c r="A27" s="23"/>
       <c r="B27" s="8"/>
       <c r="C27" s="8"/>
       <c r="D27" s="8"/>
@@ -8086,13 +8000,13 @@
       <c r="F27" s="8"/>
       <c r="G27" s="8"/>
       <c r="H27" s="8"/>
-      <c r="I27" s="82" t="s">
+      <c r="I27" s="67" t="s">
         <v>45</v>
       </c>
-      <c r="J27" s="73"/>
-      <c r="K27" s="73"/>
-      <c r="L27" s="73"/>
-      <c r="M27" s="74"/>
+      <c r="J27" s="45"/>
+      <c r="K27" s="45"/>
+      <c r="L27" s="45"/>
+      <c r="M27" s="46"/>
       <c r="N27" s="8"/>
       <c r="O27" s="8"/>
       <c r="P27" s="8"/>
@@ -8100,46 +8014,46 @@
       <c r="R27" s="8"/>
       <c r="S27" s="8"/>
       <c r="T27" s="8"/>
-      <c r="U27" s="19"/>
+      <c r="U27" s="15"/>
     </row>
     <row r="28" spans="1:21">
       <c r="A28" s="5"/>
-      <c r="I28" s="59" t="s">
+      <c r="I28" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="J28" s="59" t="s">
+      <c r="J28" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="K28" s="59" t="s">
+      <c r="K28" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="L28" s="59" t="s">
+      <c r="L28" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="M28" s="59" t="s">
+      <c r="M28" s="26" t="s">
         <v>25</v>
       </c>
       <c r="U28" s="7"/>
     </row>
     <row r="29" spans="1:21">
       <c r="A29" s="5"/>
-      <c r="I29" s="63">
+      <c r="I29" s="29">
         <f>Weely!E8</f>
         <v>0</v>
       </c>
-      <c r="J29" s="63">
+      <c r="J29" s="29">
         <f>Weely!G8</f>
         <v>0</v>
       </c>
-      <c r="K29" s="63">
+      <c r="K29" s="29">
         <f>Weely!I8</f>
         <v>0</v>
       </c>
-      <c r="L29" s="63">
+      <c r="L29" s="29">
         <f>Weely!K8</f>
         <v>0</v>
       </c>
-      <c r="M29" s="63">
+      <c r="M29" s="29">
         <f>Weely!M8</f>
         <v>0</v>
       </c>
@@ -8147,26 +8061,26 @@
     </row>
     <row r="30" spans="1:21">
       <c r="A30" s="5"/>
-      <c r="H30" s="20" t="s">
+      <c r="H30" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="I30" s="63">
+      <c r="I30" s="29">
         <f>Weely!E9</f>
         <v>0</v>
       </c>
-      <c r="J30" s="63">
+      <c r="J30" s="29">
         <f>Weely!G9</f>
         <v>0</v>
       </c>
-      <c r="K30" s="63">
+      <c r="K30" s="29">
         <f>Weely!I9</f>
         <v>0</v>
       </c>
-      <c r="L30" s="63">
+      <c r="L30" s="29">
         <f>Weely!K9</f>
         <v>0</v>
       </c>
-      <c r="M30" s="63">
+      <c r="M30" s="29">
         <f>Weely!M9</f>
         <v>0</v>
       </c>
@@ -8181,75 +8095,72 @@
     </row>
     <row r="32" spans="1:21" ht="15.6">
       <c r="A32" s="5"/>
-      <c r="D32" s="101" t="s">
+      <c r="D32" s="71" t="s">
         <v>149</v>
       </c>
-      <c r="E32" s="101"/>
-      <c r="F32" s="101"/>
-      <c r="G32" s="101"/>
-      <c r="H32" s="101"/>
-      <c r="I32" s="101"/>
-      <c r="J32" s="101"/>
+      <c r="E32" s="71"/>
+      <c r="F32" s="71"/>
+      <c r="G32" s="71"/>
+      <c r="H32" s="71"/>
+      <c r="I32" s="71"/>
+      <c r="J32" s="71"/>
       <c r="K32" s="8"/>
       <c r="L32" s="8"/>
       <c r="M32" s="8"/>
       <c r="U32" s="7"/>
     </row>
     <row r="33" spans="1:25" s="1" customFormat="1" ht="43.2" customHeight="1">
-      <c r="A33" s="70"/>
-      <c r="D33" s="69" t="s">
+      <c r="A33" s="35"/>
+      <c r="D33" s="87" t="s">
         <v>47</v>
       </c>
-      <c r="E33" s="42" t="s">
+      <c r="E33" s="82" t="s">
         <v>48</v>
       </c>
-      <c r="F33" s="42" t="s">
+      <c r="F33" s="82" t="s">
         <v>49</v>
       </c>
-      <c r="G33" s="34" t="s">
+      <c r="G33" s="82" t="s">
         <v>51</v>
       </c>
-      <c r="H33" s="43" t="s">
+      <c r="H33" s="82" t="s">
         <v>52</v>
       </c>
-      <c r="I33" s="41" t="s">
+      <c r="I33" s="82" t="s">
         <v>53</v>
       </c>
-      <c r="J33" s="57" t="s">
+      <c r="J33" s="88" t="s">
         <v>61</v>
       </c>
       <c r="U33" s="7"/>
-      <c r="V33" s="23"/>
-      <c r="W33" s="24"/>
-      <c r="X33" s="24"/>
-      <c r="Y33" s="22"/>
+      <c r="V33" s="19"/>
+      <c r="W33" s="20"/>
+      <c r="X33" s="20"/>
+      <c r="Y33" s="18"/>
     </row>
     <row r="34" spans="1:25">
       <c r="A34" s="5"/>
-      <c r="D34" s="27" t="s">
+      <c r="D34" s="31" t="s">
         <v>147</v>
       </c>
-      <c r="E34" s="25">
+      <c r="E34" s="89">
         <v>8.3000000000000007</v>
       </c>
-      <c r="F34" s="25">
+      <c r="F34" s="89">
         <v>17.3</v>
       </c>
-      <c r="G34" s="58">
+      <c r="G34" s="90">
         <v>490</v>
       </c>
-      <c r="H34" s="27">
+      <c r="H34" s="31">
         <v>10</v>
       </c>
-      <c r="I34" s="29">
+      <c r="I34" s="85">
         <v>5</v>
       </c>
-      <c r="J34" s="58" t="e">
-        <f t="shared" ref="J34" si="0">IF(#REF!&gt;0, ROUND((#REF!-#REF!)/#REF!*100, 0), 0)</f>
-        <v>#REF!</v>
-      </c>
+      <c r="J34" s="90"/>
       <c r="U34" s="7"/>
-      <c r="V34" s="21"/>
+      <c r="V34" s="17"/>
       <c r="X34" s="8"/>
     </row>
     <row r="35" spans="1:25">
@@ -8258,229 +8169,229 @@
         <v>148</v>
       </c>
       <c r="U35" s="7"/>
-      <c r="V35" s="21"/>
+      <c r="V35" s="17"/>
       <c r="X35" s="8"/>
     </row>
     <row r="36" spans="1:25">
-      <c r="A36" s="95" t="s">
+      <c r="A36" s="68" t="s">
         <v>46</v>
       </c>
-      <c r="B36" s="73"/>
-      <c r="C36" s="73"/>
-      <c r="D36" s="73"/>
-      <c r="E36" s="73"/>
-      <c r="F36" s="73"/>
-      <c r="G36" s="73"/>
-      <c r="H36" s="73"/>
-      <c r="I36" s="73"/>
-      <c r="J36" s="73"/>
-      <c r="K36" s="73"/>
-      <c r="L36" s="73"/>
-      <c r="M36" s="73"/>
-      <c r="N36" s="73"/>
-      <c r="O36" s="73"/>
-      <c r="P36" s="73"/>
-      <c r="Q36" s="73"/>
-      <c r="R36" s="73"/>
-      <c r="S36" s="73"/>
-      <c r="T36" s="73"/>
-      <c r="U36" s="96"/>
+      <c r="B36" s="45"/>
+      <c r="C36" s="45"/>
+      <c r="D36" s="45"/>
+      <c r="E36" s="45"/>
+      <c r="F36" s="45"/>
+      <c r="G36" s="45"/>
+      <c r="H36" s="45"/>
+      <c r="I36" s="45"/>
+      <c r="J36" s="45"/>
+      <c r="K36" s="45"/>
+      <c r="L36" s="45"/>
+      <c r="M36" s="45"/>
+      <c r="N36" s="45"/>
+      <c r="O36" s="45"/>
+      <c r="P36" s="45"/>
+      <c r="Q36" s="45"/>
+      <c r="R36" s="45"/>
+      <c r="S36" s="45"/>
+      <c r="T36" s="45"/>
+      <c r="U36" s="69"/>
     </row>
     <row r="37" spans="1:25" s="1" customFormat="1" ht="43.2" customHeight="1">
-      <c r="A37" s="60" t="s">
+      <c r="A37" s="81" t="s">
         <v>50</v>
       </c>
-      <c r="B37" s="34" t="s">
+      <c r="B37" s="82" t="s">
         <v>54</v>
       </c>
-      <c r="C37" s="40" t="s">
+      <c r="C37" s="82" t="s">
         <v>55</v>
       </c>
-      <c r="D37" s="40" t="s">
+      <c r="D37" s="82" t="s">
         <v>56</v>
       </c>
-      <c r="E37" s="40" t="s">
+      <c r="E37" s="82" t="s">
         <v>57</v>
       </c>
-      <c r="F37" s="40" t="s">
+      <c r="F37" s="82" t="s">
         <v>58</v>
       </c>
-      <c r="G37" s="40" t="s">
+      <c r="G37" s="82" t="s">
         <v>59</v>
       </c>
-      <c r="H37" s="97" t="s">
+      <c r="H37" s="83" t="s">
         <v>60</v>
       </c>
-      <c r="I37" s="98"/>
-      <c r="J37" s="99"/>
+      <c r="I37" s="48"/>
+      <c r="J37" s="49"/>
       <c r="U37" s="7"/>
-      <c r="V37" s="23"/>
-      <c r="W37" s="24"/>
-      <c r="X37" s="24"/>
-      <c r="Y37" s="22"/>
+      <c r="V37" s="19"/>
+      <c r="W37" s="20"/>
+      <c r="X37" s="20"/>
+      <c r="Y37" s="18"/>
     </row>
     <row r="38" spans="1:25">
-      <c r="A38" s="71" t="s">
+      <c r="A38" s="84" t="s">
         <v>62</v>
       </c>
-      <c r="B38" s="29">
+      <c r="B38" s="85">
         <v>13</v>
       </c>
-      <c r="C38" s="29">
-        <v>0</v>
-      </c>
-      <c r="D38" s="29">
+      <c r="C38" s="85">
+        <v>0</v>
+      </c>
+      <c r="D38" s="85">
         <v>7.2</v>
       </c>
-      <c r="E38" s="29">
+      <c r="E38" s="85">
         <v>5.4</v>
       </c>
-      <c r="F38" s="29">
+      <c r="F38" s="85">
         <v>14.1</v>
       </c>
-      <c r="G38" s="29">
-        <v>0</v>
-      </c>
-      <c r="H38" s="102"/>
-      <c r="I38" s="73"/>
-      <c r="J38" s="74"/>
+      <c r="G38" s="85">
+        <v>0</v>
+      </c>
+      <c r="H38" s="86"/>
+      <c r="I38" s="48"/>
+      <c r="J38" s="49"/>
       <c r="U38" s="7"/>
-      <c r="V38" s="21"/>
+      <c r="V38" s="17"/>
       <c r="X38" s="8"/>
     </row>
     <row r="39" spans="1:25">
-      <c r="A39" s="71" t="s">
+      <c r="A39" s="84" t="s">
         <v>63</v>
       </c>
-      <c r="B39" s="29">
+      <c r="B39" s="85">
         <v>12</v>
       </c>
-      <c r="C39" s="29">
-        <v>0</v>
-      </c>
-      <c r="D39" s="29">
-        <v>0</v>
-      </c>
-      <c r="E39" s="29">
-        <v>0</v>
-      </c>
-      <c r="F39" s="29">
-        <v>0</v>
-      </c>
-      <c r="G39" s="29">
-        <v>0</v>
-      </c>
-      <c r="H39" s="102"/>
-      <c r="I39" s="73"/>
-      <c r="J39" s="74"/>
+      <c r="C39" s="85">
+        <v>0</v>
+      </c>
+      <c r="D39" s="85">
+        <v>0</v>
+      </c>
+      <c r="E39" s="85">
+        <v>0</v>
+      </c>
+      <c r="F39" s="85">
+        <v>0</v>
+      </c>
+      <c r="G39" s="85">
+        <v>0</v>
+      </c>
+      <c r="H39" s="86"/>
+      <c r="I39" s="48"/>
+      <c r="J39" s="49"/>
       <c r="U39" s="7"/>
     </row>
     <row r="40" spans="1:25">
-      <c r="A40" s="71" t="s">
+      <c r="A40" s="84" t="s">
         <v>64</v>
       </c>
-      <c r="B40" s="29">
+      <c r="B40" s="85">
         <v>11</v>
       </c>
-      <c r="C40" s="29">
-        <v>0</v>
-      </c>
-      <c r="D40" s="29">
-        <v>0</v>
-      </c>
-      <c r="E40" s="29">
-        <v>0</v>
-      </c>
-      <c r="F40" s="29">
-        <v>0</v>
-      </c>
-      <c r="G40" s="29">
-        <v>0</v>
-      </c>
-      <c r="H40" s="102"/>
-      <c r="I40" s="73"/>
-      <c r="J40" s="74"/>
+      <c r="C40" s="85">
+        <v>0</v>
+      </c>
+      <c r="D40" s="85">
+        <v>0</v>
+      </c>
+      <c r="E40" s="85">
+        <v>0</v>
+      </c>
+      <c r="F40" s="85">
+        <v>0</v>
+      </c>
+      <c r="G40" s="85">
+        <v>0</v>
+      </c>
+      <c r="H40" s="86"/>
+      <c r="I40" s="48"/>
+      <c r="J40" s="49"/>
       <c r="U40" s="7"/>
     </row>
     <row r="41" spans="1:25">
-      <c r="A41" s="71" t="s">
+      <c r="A41" s="84" t="s">
         <v>65</v>
       </c>
-      <c r="B41" s="29">
+      <c r="B41" s="85">
         <v>20</v>
       </c>
-      <c r="C41" s="29">
+      <c r="C41" s="85">
         <v>67.599999999999994</v>
       </c>
-      <c r="D41" s="29">
-        <v>0</v>
-      </c>
-      <c r="E41" s="29">
-        <v>0</v>
-      </c>
-      <c r="F41" s="29">
-        <v>0</v>
-      </c>
-      <c r="G41" s="29">
-        <v>0</v>
-      </c>
-      <c r="H41" s="102"/>
-      <c r="I41" s="73"/>
-      <c r="J41" s="74"/>
+      <c r="D41" s="85">
+        <v>0</v>
+      </c>
+      <c r="E41" s="85">
+        <v>0</v>
+      </c>
+      <c r="F41" s="85">
+        <v>0</v>
+      </c>
+      <c r="G41" s="85">
+        <v>0</v>
+      </c>
+      <c r="H41" s="86"/>
+      <c r="I41" s="48"/>
+      <c r="J41" s="49"/>
       <c r="U41" s="7"/>
     </row>
     <row r="42" spans="1:25">
-      <c r="A42" s="71" t="s">
+      <c r="A42" s="84" t="s">
         <v>66</v>
       </c>
-      <c r="B42" s="29">
+      <c r="B42" s="85">
         <v>25</v>
       </c>
-      <c r="C42" s="29">
-        <v>0</v>
-      </c>
-      <c r="D42" s="29">
-        <v>0</v>
-      </c>
-      <c r="E42" s="29">
-        <v>0</v>
-      </c>
-      <c r="F42" s="29">
+      <c r="C42" s="85">
+        <v>0</v>
+      </c>
+      <c r="D42" s="85">
+        <v>0</v>
+      </c>
+      <c r="E42" s="85">
+        <v>0</v>
+      </c>
+      <c r="F42" s="85">
         <v>113.8</v>
       </c>
-      <c r="G42" s="29">
-        <v>0</v>
-      </c>
-      <c r="H42" s="102"/>
-      <c r="I42" s="73"/>
-      <c r="J42" s="74"/>
+      <c r="G42" s="85">
+        <v>0</v>
+      </c>
+      <c r="H42" s="86"/>
+      <c r="I42" s="48"/>
+      <c r="J42" s="49"/>
       <c r="U42" s="7"/>
     </row>
     <row r="43" spans="1:25">
-      <c r="A43" s="71" t="s">
+      <c r="A43" s="84" t="s">
         <v>67</v>
       </c>
-      <c r="B43" s="29">
+      <c r="B43" s="85">
         <v>55</v>
       </c>
-      <c r="C43" s="29">
+      <c r="C43" s="85">
         <v>166.7</v>
       </c>
-      <c r="D43" s="29">
-        <v>0</v>
-      </c>
-      <c r="E43" s="29">
-        <v>0</v>
-      </c>
-      <c r="F43" s="29">
-        <v>0</v>
-      </c>
-      <c r="G43" s="29">
-        <v>0</v>
-      </c>
-      <c r="H43" s="102"/>
-      <c r="I43" s="73"/>
-      <c r="J43" s="74"/>
+      <c r="D43" s="85">
+        <v>0</v>
+      </c>
+      <c r="E43" s="85">
+        <v>0</v>
+      </c>
+      <c r="F43" s="85">
+        <v>0</v>
+      </c>
+      <c r="G43" s="85">
+        <v>0</v>
+      </c>
+      <c r="H43" s="86"/>
+      <c r="I43" s="48"/>
+      <c r="J43" s="49"/>
       <c r="U43" s="7"/>
     </row>
     <row r="44" spans="1:25">
@@ -8488,392 +8399,382 @@
       <c r="U44" s="7"/>
     </row>
     <row r="45" spans="1:25">
-      <c r="A45" s="91" t="s">
+      <c r="A45" s="52" t="s">
         <v>68</v>
       </c>
-      <c r="B45" s="85"/>
-      <c r="C45" s="85"/>
-      <c r="D45" s="86"/>
-      <c r="E45" s="103">
+      <c r="B45" s="53"/>
+      <c r="C45" s="53"/>
+      <c r="D45" s="54"/>
+      <c r="E45" s="58">
         <v>46182</v>
       </c>
-      <c r="F45" s="73"/>
-      <c r="G45" s="73"/>
-      <c r="H45" s="73"/>
-      <c r="I45" s="73"/>
-      <c r="J45" s="73"/>
-      <c r="K45" s="73"/>
-      <c r="L45" s="73"/>
-      <c r="M45" s="73"/>
-      <c r="N45" s="74"/>
-      <c r="O45" s="104"/>
-      <c r="P45" s="85"/>
-      <c r="Q45" s="85"/>
-      <c r="R45" s="85"/>
-      <c r="S45" s="85"/>
-      <c r="T45" s="85"/>
-      <c r="U45" s="105"/>
+      <c r="F45" s="45"/>
+      <c r="G45" s="45"/>
+      <c r="H45" s="45"/>
+      <c r="I45" s="45"/>
+      <c r="J45" s="45"/>
+      <c r="K45" s="45"/>
+      <c r="L45" s="45"/>
+      <c r="M45" s="45"/>
+      <c r="N45" s="46"/>
+      <c r="O45" s="59"/>
+      <c r="P45" s="53"/>
+      <c r="Q45" s="53"/>
+      <c r="R45" s="53"/>
+      <c r="S45" s="53"/>
+      <c r="T45" s="53"/>
+      <c r="U45" s="60"/>
     </row>
     <row r="46" spans="1:25">
-      <c r="A46" s="87"/>
-      <c r="B46" s="88"/>
-      <c r="C46" s="88"/>
-      <c r="D46" s="89"/>
-      <c r="E46" s="108" t="s">
+      <c r="A46" s="55"/>
+      <c r="B46" s="56"/>
+      <c r="C46" s="56"/>
+      <c r="D46" s="57"/>
+      <c r="E46" s="63" t="s">
         <v>69</v>
       </c>
-      <c r="F46" s="73"/>
-      <c r="G46" s="73"/>
-      <c r="H46" s="73"/>
-      <c r="I46" s="73"/>
-      <c r="J46" s="73"/>
-      <c r="K46" s="73"/>
-      <c r="L46" s="73"/>
-      <c r="M46" s="73"/>
-      <c r="N46" s="74"/>
-      <c r="O46" s="106"/>
-      <c r="P46" s="88"/>
-      <c r="Q46" s="88"/>
-      <c r="R46" s="88"/>
-      <c r="S46" s="88"/>
-      <c r="T46" s="88"/>
-      <c r="U46" s="107"/>
+      <c r="F46" s="45"/>
+      <c r="G46" s="45"/>
+      <c r="H46" s="45"/>
+      <c r="I46" s="45"/>
+      <c r="J46" s="45"/>
+      <c r="K46" s="45"/>
+      <c r="L46" s="45"/>
+      <c r="M46" s="45"/>
+      <c r="N46" s="46"/>
+      <c r="O46" s="61"/>
+      <c r="P46" s="56"/>
+      <c r="Q46" s="56"/>
+      <c r="R46" s="56"/>
+      <c r="S46" s="56"/>
+      <c r="T46" s="56"/>
+      <c r="U46" s="62"/>
     </row>
     <row r="47" spans="1:25" s="2" customFormat="1">
-      <c r="A47" s="109" t="s">
+      <c r="A47" s="64" t="s">
         <v>70</v>
       </c>
-      <c r="B47" s="73"/>
-      <c r="C47" s="73"/>
-      <c r="D47" s="74"/>
-      <c r="E47" s="62" t="s">
+      <c r="B47" s="45"/>
+      <c r="C47" s="45"/>
+      <c r="D47" s="46"/>
+      <c r="E47" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="F47" s="62" t="s">
+      <c r="F47" s="28" t="s">
         <v>71</v>
       </c>
-      <c r="G47" s="61" t="s">
+      <c r="G47" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="H47" s="61" t="s">
+      <c r="H47" s="27" t="s">
         <v>73</v>
       </c>
-      <c r="I47" s="61" t="s">
+      <c r="I47" s="27" t="s">
         <v>74</v>
       </c>
-      <c r="J47" s="61" t="s">
+      <c r="J47" s="27" t="s">
         <v>75</v>
       </c>
-      <c r="K47" s="110" t="s">
+      <c r="K47" s="65" t="s">
         <v>76</v>
       </c>
-      <c r="L47" s="111"/>
-      <c r="M47" s="110" t="s">
+      <c r="L47" s="49"/>
+      <c r="M47" s="65" t="s">
         <v>77</v>
       </c>
-      <c r="N47" s="111"/>
-      <c r="O47" s="112" t="s">
+      <c r="N47" s="49"/>
+      <c r="O47" s="66" t="s">
         <v>78</v>
       </c>
-      <c r="P47" s="113"/>
-      <c r="Q47" s="113"/>
-      <c r="R47" s="111"/>
-      <c r="S47" s="110" t="s">
+      <c r="P47" s="48"/>
+      <c r="Q47" s="48"/>
+      <c r="R47" s="49"/>
+      <c r="S47" s="65" t="s">
         <v>79</v>
       </c>
-      <c r="T47" s="113"/>
-      <c r="U47" s="114"/>
+      <c r="T47" s="48"/>
+      <c r="U47" s="51"/>
     </row>
     <row r="48" spans="1:25">
-      <c r="A48" s="84" t="s">
+      <c r="A48" s="44" t="s">
         <v>80</v>
       </c>
-      <c r="B48" s="73"/>
-      <c r="C48" s="73"/>
-      <c r="D48" s="74"/>
-      <c r="E48" s="65">
+      <c r="B48" s="45"/>
+      <c r="C48" s="45"/>
+      <c r="D48" s="46"/>
+      <c r="E48" s="31">
         <f>'Line Stop_Prod Loss'!G5</f>
         <v>0.5</v>
       </c>
-      <c r="F48" s="65">
+      <c r="F48" s="31">
         <f>'Line Stop_Prod Loss'!H5</f>
         <v>73.7</v>
       </c>
-      <c r="G48" s="65">
+      <c r="G48" s="31">
         <f>'Line Stop_Prod Loss'!F5</f>
         <v>0</v>
       </c>
-      <c r="H48" s="65">
+      <c r="H48" s="31">
         <f>'Line Stop_Prod Loss'!E5</f>
         <v>0</v>
       </c>
-      <c r="I48" s="65">
+      <c r="I48" s="31">
         <f>'Line Stop_Prod Loss'!D5</f>
         <v>0</v>
       </c>
-      <c r="J48" s="65">
+      <c r="J48" s="31">
         <f>'Line Stop_Prod Loss'!C5</f>
         <v>0</v>
       </c>
-      <c r="K48" s="65">
-        <v>0</v>
-      </c>
-      <c r="L48" s="65">
-        <v>0</v>
-      </c>
-      <c r="M48" s="65">
-        <v>0</v>
-      </c>
-      <c r="N48" s="65">
-        <v>0</v>
-      </c>
-      <c r="O48" s="115"/>
-      <c r="P48" s="113"/>
-      <c r="Q48" s="113"/>
-      <c r="R48" s="111"/>
-      <c r="S48" s="116"/>
-      <c r="T48" s="113"/>
-      <c r="U48" s="114"/>
+      <c r="K48" s="31">
+        <v>0</v>
+      </c>
+      <c r="L48" s="31">
+        <v>0</v>
+      </c>
+      <c r="M48" s="31">
+        <v>0</v>
+      </c>
+      <c r="N48" s="31">
+        <v>0</v>
+      </c>
+      <c r="O48" s="47"/>
+      <c r="P48" s="48"/>
+      <c r="Q48" s="48"/>
+      <c r="R48" s="49"/>
+      <c r="S48" s="50"/>
+      <c r="T48" s="48"/>
+      <c r="U48" s="51"/>
     </row>
     <row r="49" spans="1:21">
-      <c r="A49" s="84" t="s">
+      <c r="A49" s="44" t="s">
         <v>82</v>
       </c>
-      <c r="B49" s="73"/>
-      <c r="C49" s="73"/>
-      <c r="D49" s="74"/>
-      <c r="E49" s="28">
+      <c r="B49" s="45"/>
+      <c r="C49" s="45"/>
+      <c r="D49" s="46"/>
+      <c r="E49" s="21">
         <f>'Line Stop_Prod Loss'!G6</f>
         <v>156.30000000000001</v>
       </c>
-      <c r="F49" s="28">
+      <c r="F49" s="21">
         <f>'Line Stop_Prod Loss'!H6</f>
         <v>0</v>
       </c>
-      <c r="G49" s="28">
+      <c r="G49" s="21">
         <f>'Line Stop_Prod Loss'!F6</f>
         <v>0</v>
       </c>
-      <c r="H49" s="28">
+      <c r="H49" s="21">
         <f>'Line Stop_Prod Loss'!E6</f>
         <v>0</v>
       </c>
-      <c r="I49" s="28">
+      <c r="I49" s="21">
         <f>'Line Stop_Prod Loss'!D6</f>
         <v>0</v>
       </c>
-      <c r="J49" s="28">
+      <c r="J49" s="21">
         <f>'Line Stop_Prod Loss'!C6</f>
         <v>0</v>
       </c>
-      <c r="K49" s="28">
-        <v>0</v>
-      </c>
-      <c r="L49" s="28">
-        <v>0</v>
-      </c>
-      <c r="M49" s="28">
-        <v>0</v>
-      </c>
-      <c r="N49" s="28">
-        <v>0</v>
-      </c>
-      <c r="O49" s="115"/>
-      <c r="P49" s="113"/>
-      <c r="Q49" s="113"/>
-      <c r="R49" s="111"/>
-      <c r="S49" s="116"/>
-      <c r="T49" s="113"/>
-      <c r="U49" s="114"/>
+      <c r="K49" s="21">
+        <v>0</v>
+      </c>
+      <c r="L49" s="21">
+        <v>0</v>
+      </c>
+      <c r="M49" s="21">
+        <v>0</v>
+      </c>
+      <c r="N49" s="21">
+        <v>0</v>
+      </c>
+      <c r="O49" s="47"/>
+      <c r="P49" s="48"/>
+      <c r="Q49" s="48"/>
+      <c r="R49" s="49"/>
+      <c r="S49" s="50"/>
+      <c r="T49" s="48"/>
+      <c r="U49" s="51"/>
     </row>
     <row r="50" spans="1:21">
-      <c r="A50" s="84" t="s">
+      <c r="A50" s="44" t="s">
         <v>84</v>
       </c>
-      <c r="B50" s="73"/>
-      <c r="C50" s="73"/>
-      <c r="D50" s="74"/>
-      <c r="E50" s="28">
+      <c r="B50" s="45"/>
+      <c r="C50" s="45"/>
+      <c r="D50" s="46"/>
+      <c r="E50" s="21">
         <f>'Line Stop_Prod Loss'!G7</f>
         <v>0</v>
       </c>
-      <c r="F50" s="28">
+      <c r="F50" s="21">
         <f>'Line Stop_Prod Loss'!H7</f>
         <v>0.2</v>
       </c>
-      <c r="G50" s="28">
+      <c r="G50" s="21">
         <f>'Line Stop_Prod Loss'!F7</f>
         <v>0</v>
       </c>
-      <c r="H50" s="28">
+      <c r="H50" s="21">
         <f>'Line Stop_Prod Loss'!E7</f>
         <v>0</v>
       </c>
-      <c r="I50" s="28">
+      <c r="I50" s="21">
         <f>'Line Stop_Prod Loss'!D7</f>
         <v>0</v>
       </c>
-      <c r="J50" s="28">
+      <c r="J50" s="21">
         <f>'Line Stop_Prod Loss'!C7</f>
         <v>0</v>
       </c>
-      <c r="K50" s="28">
-        <v>0</v>
-      </c>
-      <c r="L50" s="28">
-        <v>0</v>
-      </c>
-      <c r="M50" s="28">
-        <v>0</v>
-      </c>
-      <c r="N50" s="28">
-        <v>0</v>
-      </c>
-      <c r="O50" s="115"/>
-      <c r="P50" s="113"/>
-      <c r="Q50" s="113"/>
-      <c r="R50" s="111"/>
-      <c r="S50" s="116"/>
-      <c r="T50" s="113"/>
-      <c r="U50" s="114"/>
+      <c r="K50" s="21">
+        <v>0</v>
+      </c>
+      <c r="L50" s="21">
+        <v>0</v>
+      </c>
+      <c r="M50" s="21">
+        <v>0</v>
+      </c>
+      <c r="N50" s="21">
+        <v>0</v>
+      </c>
+      <c r="O50" s="47"/>
+      <c r="P50" s="48"/>
+      <c r="Q50" s="48"/>
+      <c r="R50" s="49"/>
+      <c r="S50" s="50"/>
+      <c r="T50" s="48"/>
+      <c r="U50" s="51"/>
     </row>
     <row r="51" spans="1:21">
-      <c r="A51" s="84" t="s">
+      <c r="A51" s="44" t="s">
         <v>85</v>
       </c>
-      <c r="B51" s="73"/>
-      <c r="C51" s="73"/>
-      <c r="D51" s="74"/>
-      <c r="E51" s="28">
+      <c r="B51" s="45"/>
+      <c r="C51" s="45"/>
+      <c r="D51" s="46"/>
+      <c r="E51" s="21">
         <f>'Line Stop_Prod Loss'!G8</f>
         <v>0.1</v>
       </c>
-      <c r="F51" s="28">
+      <c r="F51" s="21">
         <f>'Line Stop_Prod Loss'!H8</f>
         <v>0.1</v>
       </c>
-      <c r="G51" s="28">
+      <c r="G51" s="21">
         <f>'Line Stop_Prod Loss'!F8</f>
         <v>0</v>
       </c>
-      <c r="H51" s="28">
+      <c r="H51" s="21">
         <f>'Line Stop_Prod Loss'!E8</f>
         <v>0</v>
       </c>
-      <c r="I51" s="28">
+      <c r="I51" s="21">
         <f>'Line Stop_Prod Loss'!D8</f>
         <v>0</v>
       </c>
-      <c r="J51" s="28">
+      <c r="J51" s="21">
         <f>'Line Stop_Prod Loss'!C8</f>
         <v>0</v>
       </c>
-      <c r="K51" s="28">
-        <v>0</v>
-      </c>
-      <c r="L51" s="28">
-        <v>0</v>
-      </c>
-      <c r="M51" s="28">
-        <v>0</v>
-      </c>
-      <c r="N51" s="28">
-        <v>0</v>
-      </c>
-      <c r="O51" s="115"/>
-      <c r="P51" s="113"/>
-      <c r="Q51" s="113"/>
-      <c r="R51" s="111"/>
-      <c r="S51" s="116"/>
-      <c r="T51" s="113"/>
-      <c r="U51" s="114"/>
+      <c r="K51" s="21">
+        <v>0</v>
+      </c>
+      <c r="L51" s="21">
+        <v>0</v>
+      </c>
+      <c r="M51" s="21">
+        <v>0</v>
+      </c>
+      <c r="N51" s="21">
+        <v>0</v>
+      </c>
+      <c r="O51" s="47"/>
+      <c r="P51" s="48"/>
+      <c r="Q51" s="48"/>
+      <c r="R51" s="49"/>
+      <c r="S51" s="50"/>
+      <c r="T51" s="48"/>
+      <c r="U51" s="51"/>
     </row>
     <row r="52" spans="1:21" ht="15" customHeight="1" thickBot="1">
-      <c r="A52" s="117" t="s">
+      <c r="A52" s="36" t="s">
         <v>87</v>
       </c>
-      <c r="B52" s="118"/>
-      <c r="C52" s="118"/>
-      <c r="D52" s="119"/>
-      <c r="E52" s="68">
+      <c r="B52" s="37"/>
+      <c r="C52" s="37"/>
+      <c r="D52" s="38"/>
+      <c r="E52" s="34">
         <f>'Line Stop_Prod Loss'!G9</f>
         <v>0</v>
       </c>
-      <c r="F52" s="68">
+      <c r="F52" s="34">
         <f>'Line Stop_Prod Loss'!H9</f>
         <v>0</v>
       </c>
-      <c r="G52" s="68">
+      <c r="G52" s="34">
         <f>'Line Stop_Prod Loss'!F9</f>
         <v>0</v>
       </c>
-      <c r="H52" s="68">
+      <c r="H52" s="34">
         <f>'Line Stop_Prod Loss'!E9</f>
         <v>0</v>
       </c>
-      <c r="I52" s="68">
+      <c r="I52" s="34">
         <f>'Line Stop_Prod Loss'!D9</f>
         <v>0</v>
       </c>
-      <c r="J52" s="68">
+      <c r="J52" s="34">
         <f>'Line Stop_Prod Loss'!C9</f>
         <v>0</v>
       </c>
-      <c r="K52" s="68">
-        <v>0</v>
-      </c>
-      <c r="L52" s="68">
-        <v>0</v>
-      </c>
-      <c r="M52" s="68">
-        <v>0</v>
-      </c>
-      <c r="N52" s="68">
-        <v>0</v>
-      </c>
-      <c r="O52" s="120"/>
-      <c r="P52" s="121"/>
-      <c r="Q52" s="121"/>
-      <c r="R52" s="122"/>
-      <c r="S52" s="123"/>
-      <c r="T52" s="121"/>
-      <c r="U52" s="124"/>
+      <c r="K52" s="34">
+        <v>0</v>
+      </c>
+      <c r="L52" s="34">
+        <v>0</v>
+      </c>
+      <c r="M52" s="34">
+        <v>0</v>
+      </c>
+      <c r="N52" s="34">
+        <v>0</v>
+      </c>
+      <c r="O52" s="39"/>
+      <c r="P52" s="40"/>
+      <c r="Q52" s="40"/>
+      <c r="R52" s="41"/>
+      <c r="S52" s="42"/>
+      <c r="T52" s="40"/>
+      <c r="U52" s="43"/>
     </row>
     <row r="53" spans="1:21">
       <c r="L53" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="64">
-    <mergeCell ref="A52:D52"/>
-    <mergeCell ref="O52:R52"/>
-    <mergeCell ref="S52:U52"/>
-    <mergeCell ref="A50:D50"/>
-    <mergeCell ref="O50:R50"/>
-    <mergeCell ref="S50:U50"/>
-    <mergeCell ref="A51:D51"/>
-    <mergeCell ref="O51:R51"/>
-    <mergeCell ref="S51:U51"/>
-    <mergeCell ref="A48:D48"/>
-    <mergeCell ref="O48:R48"/>
-    <mergeCell ref="S48:U48"/>
-    <mergeCell ref="A49:D49"/>
-    <mergeCell ref="O49:R49"/>
-    <mergeCell ref="S49:U49"/>
-    <mergeCell ref="A45:D46"/>
-    <mergeCell ref="E45:N45"/>
-    <mergeCell ref="O45:U46"/>
-    <mergeCell ref="E46:N46"/>
-    <mergeCell ref="A47:D47"/>
-    <mergeCell ref="K47:L47"/>
-    <mergeCell ref="M47:N47"/>
-    <mergeCell ref="O47:R47"/>
-    <mergeCell ref="S47:U47"/>
-    <mergeCell ref="H42:J42"/>
-    <mergeCell ref="H43:J43"/>
-    <mergeCell ref="H40:J40"/>
-    <mergeCell ref="H41:J41"/>
-    <mergeCell ref="H38:J38"/>
-    <mergeCell ref="H39:J39"/>
+    <mergeCell ref="P6:T6"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="A1:U2"/>
+    <mergeCell ref="P4:T4"/>
+    <mergeCell ref="P5:T5"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="A8:D9"/>
+    <mergeCell ref="E8:G8"/>
+    <mergeCell ref="I8:M8"/>
+    <mergeCell ref="N8:P8"/>
+    <mergeCell ref="Q8:S8"/>
+    <mergeCell ref="E9:G9"/>
+    <mergeCell ref="I9:M9"/>
+    <mergeCell ref="N9:P9"/>
+    <mergeCell ref="Q9:S9"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="A14:D14"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="I27:M27"/>
     <mergeCell ref="A36:U36"/>
@@ -8888,26 +8789,36 @@
     <mergeCell ref="A15:B15"/>
     <mergeCell ref="C15:D15"/>
     <mergeCell ref="D32:J32"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="A13:D13"/>
-    <mergeCell ref="A14:D14"/>
-    <mergeCell ref="A8:D9"/>
-    <mergeCell ref="E8:G8"/>
-    <mergeCell ref="I8:M8"/>
-    <mergeCell ref="N8:P8"/>
-    <mergeCell ref="Q8:S8"/>
-    <mergeCell ref="E9:G9"/>
-    <mergeCell ref="I9:M9"/>
-    <mergeCell ref="N9:P9"/>
-    <mergeCell ref="Q9:S9"/>
-    <mergeCell ref="P6:T6"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="A1:U2"/>
-    <mergeCell ref="P4:T4"/>
-    <mergeCell ref="P5:T5"/>
-    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="H42:J42"/>
+    <mergeCell ref="H43:J43"/>
+    <mergeCell ref="H40:J40"/>
+    <mergeCell ref="H41:J41"/>
+    <mergeCell ref="H38:J38"/>
+    <mergeCell ref="H39:J39"/>
+    <mergeCell ref="A45:D46"/>
+    <mergeCell ref="E45:N45"/>
+    <mergeCell ref="O45:U46"/>
+    <mergeCell ref="E46:N46"/>
+    <mergeCell ref="A47:D47"/>
+    <mergeCell ref="K47:L47"/>
+    <mergeCell ref="M47:N47"/>
+    <mergeCell ref="O47:R47"/>
+    <mergeCell ref="S47:U47"/>
+    <mergeCell ref="A48:D48"/>
+    <mergeCell ref="O48:R48"/>
+    <mergeCell ref="S48:U48"/>
+    <mergeCell ref="A49:D49"/>
+    <mergeCell ref="O49:R49"/>
+    <mergeCell ref="S49:U49"/>
+    <mergeCell ref="A52:D52"/>
+    <mergeCell ref="O52:R52"/>
+    <mergeCell ref="S52:U52"/>
+    <mergeCell ref="A50:D50"/>
+    <mergeCell ref="O50:R50"/>
+    <mergeCell ref="S50:U50"/>
+    <mergeCell ref="A51:D51"/>
+    <mergeCell ref="O51:R51"/>
+    <mergeCell ref="S51:U51"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="49" orientation="landscape" r:id="rId1"/>

</xml_diff>